<commit_message>
Complement MoC workbook with BRD BO-61 B.3 requirements
Adds BRD-driven fields (ownership, scope, temporary extensions, emergency
regularisation, post-MoC verification), action handlers AH16-AH17,
workflow gate notes and decisions recording deviations from the
approved BRD. Guide updated with BRD traceability.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018d6Sqji3PhM1w1Xd54RvCw
</commit_message>
<xml_diff>
--- a/docs/moc/Impala - Configuration Workbook - Management of Change v1.2 (Impala requirements DRAFT).xlsx
+++ b/docs/moc/Impala - Configuration Workbook - Management of Change v1.2 (Impala requirements DRAFT).xlsx
@@ -28962,8 +28962,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DecisionsTasks" displayName="DecisionsTasks" ref="A4:E20" totalsRowCount="1" headerRowDxfId="1946" headerRowBorderDxfId="1945">
-  <autoFilter ref="A4:E19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DecisionsTasks" displayName="DecisionsTasks" ref="A4:E25" totalsRowCount="1" headerRowDxfId="1946" headerRowBorderDxfId="1945">
+  <autoFilter ref="A4:E24" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" totalsRowLabel="Totals" dataDxfId="1944"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Task or Decision" totalsRowFunction="count" totalsRowDxfId="1943"/>
@@ -29233,8 +29233,8 @@
 </file>
 
 <file path=xl/tables/table33.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF13000000}" name="Table6" displayName="Table6" ref="A4:F21" totalsRowCount="1" headerRowDxfId="1481" dataDxfId="1479" headerRowBorderDxfId="1480" dataCellStyle="20% - Accent1">
-  <autoFilter ref="A4:F20" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF13000000}" name="Table6" displayName="Table6" ref="A4:F23" totalsRowCount="1" headerRowDxfId="1481" dataDxfId="1479" headerRowBorderDxfId="1480" dataCellStyle="20% - Accent1">
+  <autoFilter ref="A4:F22" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-1300-000001000000}" name="#" totalsRowLabel="Total" dataDxfId="1478" totalsRowDxfId="1477" dataCellStyle="20% - Accent1"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-1300-000002000000}" name="Object Name" dataDxfId="1476" totalsRowDxfId="1475" dataCellStyle="20% - Accent1"/>
@@ -30016,7 +30016,7 @@
       <c r="F27" s="165"/>
       <c r="G27" s="165"/>
     </row>
-    <row r="28" ht="57.6" thickBot="1" x14ac:dyDescent="0.6" customHeight="1">
+    <row r="28" ht="72.0" thickBot="1" x14ac:dyDescent="0.6" customHeight="1">
       <c r="B28" s="212">
         <v>1.2</v>
       </c>
@@ -30030,7 +30030,7 @@
       </c>
       <c r="E28" s="214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala requirements - DRAFT for Design Workshop (27-Oct-2026). Sources: ILX App Overview 19-Oct-2026, Impala internal pre-design 20-Oct-2026, 'MOC Proposal.xlsx', SOW v1.5. Changes flagged A/R/M, highlighted in yellow, rationale in 'Impala Notes' columns. Open points marked [TBC].</t>
+          <t xml:space="preserve">Impala requirements - DRAFT for Design Workshop (27-Oct-2026). Sources: ILX App Overview 19-Oct-2026, Impala internal pre-design 20-Oct-2026, 'MOC Proposal.xlsx' (priority), BRD BO-61 v2.0 B.3 (complementary), SOW v1.5. Changes flagged A/R/M, highlighted in yellow, rationale in 'Impala Notes' columns. Open points marked [TBC].</t>
         </is>
       </c>
       <c r="F28" s="214" t="inlineStr">
@@ -30086,7 +30086,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <sheetPr codeName="Sheet10"/>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="6.1015625" customWidth="1"/>
@@ -30534,18 +30534,94 @@
         </is>
       </c>
     </row>
-    <row r="21" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="159" t="s">
+    <row r="21" ht="43.2" customHeight="1">
+      <c r="A21" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AH16</t>
+        </is>
+      </c>
+      <c r="B21" s="272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="C21" s="272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temporary change extension limit</t>
+        </is>
+      </c>
+      <c r="D21" s="272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max 3 extensions (BRD RULE-B3-08).</t>
+        </is>
+      </c>
+      <c r="E21" s="272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Create, Update</t>
+        </is>
+      </c>
+      <c r="F21" s="273" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If NumberOfExtensions &gt; 3
+• then error: 'A temporary change cannot be extended more than 3 times - raise a permanent MOC.'</t>
+        </is>
+      </c>
+      <c r="G21" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A - Impala requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="43.2" customHeight="1">
+      <c r="A22" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AH17</t>
+        </is>
+      </c>
+      <c r="B22" s="272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="C22" s="272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emergency regularisation gate</t>
+        </is>
+      </c>
+      <c r="D22" s="272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emergency MOC cannot close until regularised (BRD RULE-B3-14).</t>
+        </is>
+      </c>
+      <c r="E22" s="272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Update</t>
+        </is>
+      </c>
+      <c r="F22" s="273" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If EmergencyChange = Yes and action = Close and (unanswered screening questions or open tasks)
+• then error: 'Complete the retrospective MOC dossier before closing.'</t>
+        </is>
+      </c>
+      <c r="G22" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A - Impala requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23" s="159" t="s">
         <v>76</v>
       </c>
-      <c r="B21" s="159"/>
-      <c r="C21" s="160">
+      <c r="B23" s="159"/>
+      <c r="C23" s="160">
         <f>SUBTOTAL(103,Table6[Action Handler Name])</f>
         <v>13</v>
       </c>
-      <c r="D21" s="159"/>
-      <c r="E21" s="159"/>
-      <c r="F21" s="159"/>
+      <c r="D23" s="159"/>
+      <c r="E23" s="159"/>
+      <c r="F23" s="159"/>
     </row>
   </sheetData>
   <dataConsolidate/>
@@ -36391,7 +36467,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultColWidth="29.5234375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -36744,15 +36820,120 @@
       </c>
       <c r="E19" s="52"/>
     </row>
-    <row r="20" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" t="s">
+    <row r="20" ht="72.0" customHeight="1">
+      <c r="A20" s="217">
+        <v>16</v>
+      </c>
+      <c r="B20" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ratify deviations from approved BRD BO-61 v2.0 (B.3)</t>
+        </is>
+      </c>
+      <c r="C20" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Impala - Shaun Jones (MoC Process Owner)</t>
+        </is>
+      </c>
+      <c r="D20" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The 20-Oct design prevails but deviates from the approved BRD: (a) Level 0-5 scoring (FR-B3-006, RULE-B3-04) replaced by Type x Grade; (b) like-for-like exclusions not recorded in the system (FR-B3-002, Must) - rationale kept in the procedure; (c) Minor = single Terminal Manager approval vs RULE-B3-06 minimum of 2 approvers for Levels 0-3. Update Requirements Register BO61-203 and procedure CO-HS-GEN-PRO-002.</t>
+        </is>
+      </c>
+      <c r="E20" s="52"/>
+    </row>
+    <row r="21" ht="43.2" customHeight="1">
+      <c r="A21" s="217">
+        <v>17</v>
+      </c>
+      <c r="B21" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Return for revision vs formal rejection</t>
+        </is>
+      </c>
+      <c r="C21" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intelex - Ian</t>
+        </is>
+      </c>
+      <c r="D21" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-035 (Must): Roll Back from Approval = return for revision, closed approvals are KEPT; formal rejection resets the approval chain (RULE-B3-07). Intelex to confirm OOTB behaviour of approvals on Roll Back.</t>
+        </is>
+      </c>
+      <c r="E21" s="52"/>
+    </row>
+    <row r="22" ht="43.2" customHeight="1">
+      <c r="A22" s="217">
+        <v>18</v>
+      </c>
+      <c r="B22" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emergency MOC regularisation</t>
+        </is>
+      </c>
+      <c r="C22" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Impala - Shaun Jones</t>
+        </is>
+      </c>
+      <c r="D22" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD RULE-B3-14: single senior approval, immediate execution, full dossier (checklist, tasks) completed retrospectively within [TBC] days; record flagged 'pending regularisation' and reported overdue; cannot be closed until regularised (AH17).</t>
+        </is>
+      </c>
+      <c r="E22" s="52"/>
+    </row>
+    <row r="23" ht="43.2" customHeight="1">
+      <c r="A23" s="217">
+        <v>19</v>
+      </c>
+      <c r="B23" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temporary change extensions</t>
+        </is>
+      </c>
+      <c r="C23" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Impala - Sam Robinson</t>
+        </is>
+      </c>
+      <c r="D23" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD RULE-B3-08 / FR-B3-014: review date, max 3 extensions each with rationale and re-approval at the MOC grade (ad hoc approval); conversion to permanent = new MOC linked through Related MOCs.</t>
+        </is>
+      </c>
+      <c r="E23" s="52"/>
+    </row>
+    <row r="24" ht="43.2" customHeight="1">
+      <c r="A24" s="217">
+        <v>20</v>
+      </c>
+      <c r="B24" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MoC KPIs and leadership reporting</t>
+        </is>
+      </c>
+      <c r="C24" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Impala - Rodrigo Llamas</t>
+        </is>
+      </c>
+      <c r="D24" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-019 / FR-B3-033: monthly YTD permanent/temporary MOCs, open MOCs, overdue temporary MOCs, MoC-related incidents, open MoC actions + leading indicators. To be built as reports/dashboards (reporting phase), fields already captured in this workbook.</t>
+        </is>
+      </c>
+      <c r="E24" s="52"/>
+    </row>
+    <row r="25" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25" t="s">
         <v>77</v>
       </c>
-      <c r="B20" s="29">
+      <c r="B25" s="29">
         <f>SUBTOTAL(103,DecisionsTasks[Task or Decision])</f>
         <v>2</v>
       </c>
-      <c r="E20" s="29">
+      <c r="E25" s="29">
         <f>SUBTOTAL(103,DecisionsTasks[Date Complete])</f>
         <v>0</v>
       </c>
@@ -37012,7 +37193,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="158.4" x14ac:dyDescent="0.55000000000000004" customHeight="1">
+    <row r="72" ht="187.2" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A72" s="136">
         <v>3</v>
       </c>
@@ -37056,7 +37237,8 @@
 - Major: Local &gt; Regional &gt; Global HSEC + Global Operations [TBC Regional step for Major]
 Approvals are SEQUENTIAL: next level requested only when the previous level is closed (Intelex to confirm solution).
 Ad hoc approvers can be added by the MOC Coordinator.
-Prior to transitioning: at least one approval exists and all approvals are closed (accepted).</t>
+Prior to transitioning: at least one approval exists and all approvals are closed (accepted).
+Roll Back = return for revision, closed approvals are kept; a formal rejection resets the chain (BRD FR-B3-035) [Intelex to confirm].</t>
         </is>
       </c>
       <c r="J72" s="239" t="inlineStr">
@@ -37108,7 +37290,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="28.8" x14ac:dyDescent="0.55000000000000004" customHeight="1">
+    <row r="75" ht="72.0" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A75" s="139">
         <v>4</v>
       </c>
@@ -37142,7 +37324,8 @@
       <c r="I75" s="223" t="inlineStr">
         <is>
           <t xml:space="preserve">Recipient(s): Change Requester
-Prior to transitioning to next stage, all tasks have to be completed.</t>
+Prior to transitioning to next stage, all tasks have to be completed.
+Tasks of this stage = pre-startup actions (incl. PSSR where required by Type/Grade): Start Up is blocked until they are closed (BRD FR-B3-028 / FR-B3-032). Post-startup actions are created in Follow Up.</t>
         </is>
       </c>
     </row>
@@ -37268,7 +37451,7 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="72.0" x14ac:dyDescent="0.55000000000000004" customHeight="1">
+    <row r="81" ht="129.6" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A81" s="139">
         <v>6</v>
       </c>
@@ -37304,7 +37487,9 @@
           <t xml:space="preserve">Recipient(s): Change Requester
 Prior to closing:
 - All tasks and approvals have to be completed.
-- If 'Temporary Change' = Yes, then 'Has Temporary Change been scheduled for permanent MOC?' must be 'Yes' (or temporary change removed).</t>
+- If 'Temporary Change' = Yes, then 'Has Temporary Change been scheduled for permanent MOC?' must be 'Yes' (or temporary change removed).
+- If 'Emergency Change' = Yes: all screening questions answered and tasks closed (retrospective regularisation, BRD RULE-B3-14).
+- Post-MoC verification fields completed (field check, communication, downstream impacts).</t>
         </is>
       </c>
     </row>
@@ -38716,7 +38901,7 @@
         </is>
       </c>
     </row>
-    <row r="9" x14ac:dyDescent="0.55000000000000004" ht="14.4" customHeight="1">
+    <row r="9" x14ac:dyDescent="0.55000000000000004" ht="28.8" customHeight="1">
       <c r="A9" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">Regional Operations Manager</t>
@@ -38744,11 +38929,11 @@
       </c>
       <c r="F9" s="250" t="inlineStr">
         <is>
-          <t xml:space="preserve">A - Regional approval level.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="14.4" customHeight="1">
+          <t xml:space="preserve">A - Regional approval level. BRD FR-B3-007: ROM / Country Operations Manager.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28.8" customHeight="1">
       <c r="A10" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">Global HSEC</t>
@@ -38776,11 +38961,11 @@
       </c>
       <c r="F10" s="250" t="inlineStr">
         <is>
-          <t xml:space="preserve">A - Global approval level (assigned at top location).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" x14ac:dyDescent="0.55000000000000004" ht="14.4" customHeight="1">
+          <t xml:space="preserve">A - Global approval level (assigned at top location). BRD FR-B3-007: Head of HSEQ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" x14ac:dyDescent="0.55000000000000004" ht="28.8" customHeight="1">
       <c r="A11" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">Global Operations</t>
@@ -38808,7 +38993,7 @@
       </c>
       <c r="F11" s="250" t="inlineStr">
         <is>
-          <t xml:space="preserve">A - Global approval level (assigned at top location).</t>
+          <t xml:space="preserve">A - Global approval level (assigned at top location). BRD FR-B3-007: COO.</t>
         </is>
       </c>
     </row>
@@ -40072,7 +40257,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet9"/>
-  <dimension ref="A1:AC341"/>
+  <dimension ref="A1:AC354"/>
   <sheetFormatPr defaultColWidth="26.41796875" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="2.89453125" style="64" customWidth="1"/>
@@ -56899,6 +57084,1575 @@
       <c r="AA341" s="256" t="inlineStr">
         <is>
           <t xml:space="preserve">Alonso / Sam: traceability of actions back to the MOC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="342" ht="57.6" customHeight="1">
+      <c r="A342" s="253">
+        <v>10</v>
+      </c>
+      <c r="B342" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation</t>
+        </is>
+      </c>
+      <c r="C342" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D342" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation Information Details</t>
+        </is>
+      </c>
+      <c r="E342" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Change Owner</t>
+        </is>
+      </c>
+      <c r="F342" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Change Owner</t>
+        </is>
+      </c>
+      <c r="G342" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Accountable for the change through to closure.</t>
+        </is>
+      </c>
+      <c r="H342" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Relations</t>
+        </is>
+      </c>
+      <c r="I342" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tooltip: Person accountable for the change until closure (may be the requester).</t>
+        </is>
+      </c>
+      <c r="J342" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M:1 relation to Employee. Default Value: Change Requester.</t>
+        </is>
+      </c>
+      <c r="K342" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L342" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M342" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="N342" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="O342" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P342" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q342" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R342" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="S342" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T342" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="U342" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V342" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="W342" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="X342" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="AA342" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-026 (Should) / FR-B3-004: originator vs owner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="343" ht="43.2" customHeight="1">
+      <c r="A343" s="253">
+        <v>11</v>
+      </c>
+      <c r="B343" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation</t>
+        </is>
+      </c>
+      <c r="C343" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D343" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation Information Details</t>
+        </is>
+      </c>
+      <c r="E343" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operational Owner</t>
+        </is>
+      </c>
+      <c r="F343" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operational Owner</t>
+        </is>
+      </c>
+      <c r="G343" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner of the affected area or asset.</t>
+        </is>
+      </c>
+      <c r="H343" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Relations</t>
+        </is>
+      </c>
+      <c r="I343" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tooltip: Responsible for operational readiness before start-up.</t>
+        </is>
+      </c>
+      <c r="J343" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M:1 relation to Employee.</t>
+        </is>
+      </c>
+      <c r="K343" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L343" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M343" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="N343" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="O343" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P343" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q343" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R343" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="S343" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T343" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="U343" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V343" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="W343" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="X343" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="AA343" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-004 (Must).</t>
+        </is>
+      </c>
+    </row>
+    <row r="344" ht="57.6" customHeight="1">
+      <c r="A344" s="253">
+        <v>12</v>
+      </c>
+      <c r="B344" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation</t>
+        </is>
+      </c>
+      <c r="C344" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D344" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation Information Details</t>
+        </is>
+      </c>
+      <c r="E344" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reason for Change &amp; Technical Basis</t>
+        </is>
+      </c>
+      <c r="F344" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reason for Change &amp; Technical Basis</t>
+        </is>
+      </c>
+      <c r="G344" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detailed justification.</t>
+        </is>
+      </c>
+      <c r="H344" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text (multi-line)</t>
+        </is>
+      </c>
+      <c r="I344" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tooltip: Why the change is needed, technical basis, scope and current situation.</t>
+        </is>
+      </c>
+      <c r="J344" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No length limit.</t>
+        </is>
+      </c>
+      <c r="K344" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L344" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M344" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="N344" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="O344" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P344" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q344" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R344" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="S344" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T344" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="U344" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V344" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="W344" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="X344" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="AA344" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-001 (Must); Change Description is limited to 255 characters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="345" ht="28.8" customHeight="1">
+      <c r="A345" s="253">
+        <v>13</v>
+      </c>
+      <c r="B345" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation</t>
+        </is>
+      </c>
+      <c r="C345" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D345" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation Information Details</t>
+        </is>
+      </c>
+      <c r="E345" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affected Equipment / Process / System</t>
+        </is>
+      </c>
+      <c r="F345" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affected Equipment / Process / System</t>
+        </is>
+      </c>
+      <c r="G345" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What the change touches.</t>
+        </is>
+      </c>
+      <c r="H345" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="I345" s="254"/>
+      <c r="J345" s="256"/>
+      <c r="K345" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L345" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M345" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="N345" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="O345" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P345" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q345" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R345" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="S345" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T345" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="U345" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V345" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="W345" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="X345" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="AA345" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-001 (Must).</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="57.6" customHeight="1">
+      <c r="A346" s="253">
+        <v>14</v>
+      </c>
+      <c r="B346" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation</t>
+        </is>
+      </c>
+      <c r="C346" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D346" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation Information Details</t>
+        </is>
+      </c>
+      <c r="E346" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temporary Change Review Date</t>
+        </is>
+      </c>
+      <c r="F346" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temporary Change Review Date</t>
+        </is>
+      </c>
+      <c r="G346" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Next review of the temporary change.</t>
+        </is>
+      </c>
+      <c r="H346" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date</t>
+        </is>
+      </c>
+      <c r="I346" s="254"/>
+      <c r="J346" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visible and mandatory if Temporary Change = Yes. Must be on or before Change Expiry.</t>
+        </is>
+      </c>
+      <c r="K346" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L346" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M346" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="N346" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="O346" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P346" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q346" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R346" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="S346" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T346" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="U346" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V346" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="W346" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="X346" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="AA346" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-003 / FR-B3-014 (Must).</t>
+        </is>
+      </c>
+    </row>
+    <row r="347" ht="43.2" customHeight="1">
+      <c r="A347" s="253">
+        <v>15</v>
+      </c>
+      <c r="B347" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow Up</t>
+        </is>
+      </c>
+      <c r="C347" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D347" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow-Up Details</t>
+        </is>
+      </c>
+      <c r="E347" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number of Extensions</t>
+        </is>
+      </c>
+      <c r="F347" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number of Extensions</t>
+        </is>
+      </c>
+      <c r="G347" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Times the temporary change has been extended.</t>
+        </is>
+      </c>
+      <c r="H347" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number</t>
+        </is>
+      </c>
+      <c r="I347" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tooltip: Each extension needs a rationale and re-approval at the MOC grade.</t>
+        </is>
+      </c>
+      <c r="J347" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visible if Temporary Change = Yes. Max 3 (AH16).</t>
+        </is>
+      </c>
+      <c r="K347" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L347" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M347" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="N347" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="O347" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P347" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q347" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R347" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="S347" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T347" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="U347" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V347" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="W347" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="X347" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="AA347" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD RULE-B3-08 (Must).</t>
+        </is>
+      </c>
+    </row>
+    <row r="348" ht="28.8" customHeight="1">
+      <c r="A348" s="253">
+        <v>16</v>
+      </c>
+      <c r="B348" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow Up</t>
+        </is>
+      </c>
+      <c r="C348" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D348" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow-Up Details</t>
+        </is>
+      </c>
+      <c r="E348" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extension Rationale</t>
+        </is>
+      </c>
+      <c r="F348" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extension Rationale</t>
+        </is>
+      </c>
+      <c r="G348" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Why the temporary change is extended.</t>
+        </is>
+      </c>
+      <c r="H348" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="I348" s="254"/>
+      <c r="J348" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visible and mandatory if Number of Extensions &gt; 0.</t>
+        </is>
+      </c>
+      <c r="K348" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L348" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M348" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="N348" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="O348" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P348" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q348" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R348" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="S348" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T348" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="U348" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V348" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="W348" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="X348" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="AA348" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-003 (Must).</t>
+        </is>
+      </c>
+    </row>
+    <row r="349" ht="57.6" customHeight="1">
+      <c r="A349" s="253">
+        <v>17</v>
+      </c>
+      <c r="B349" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation</t>
+        </is>
+      </c>
+      <c r="C349" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D349" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Initiation Information Details</t>
+        </is>
+      </c>
+      <c r="E349" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regularisation Due Date</t>
+        </is>
+      </c>
+      <c r="F349" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Regularisation Due Date</t>
+        </is>
+      </c>
+      <c r="G349" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deadline to complete the emergency MOC dossier.</t>
+        </is>
+      </c>
+      <c r="H349" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date (calculated, read-only)</t>
+        </is>
+      </c>
+      <c r="I349" s="254"/>
+      <c r="J349" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visible if Emergency Change = Yes. = date of approval + [TBC] days. Overdue flag in reports.</t>
+        </is>
+      </c>
+      <c r="K349" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L349" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M349" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="N349" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="O349" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P349" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="Q349" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R349" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="S349" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T349" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="U349" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V349" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="W349" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="X349" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="AA349" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD RULE-B3-14 / FR-B3-015 (Must).</t>
+        </is>
+      </c>
+    </row>
+    <row r="350" ht="28.8" customHeight="1">
+      <c r="A350" s="253">
+        <v>18</v>
+      </c>
+      <c r="B350" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evaluation, Design &amp; Analysis</t>
+        </is>
+      </c>
+      <c r="C350" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D350" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evaluation, Design &amp; Analysis Details</t>
+        </is>
+      </c>
+      <c r="E350" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proposed Implementation Plan</t>
+        </is>
+      </c>
+      <c r="F350" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proposed Implementation Plan</t>
+        </is>
+      </c>
+      <c r="G350" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How and when the change will be implemented.</t>
+        </is>
+      </c>
+      <c r="H350" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text (multi-line)</t>
+        </is>
+      </c>
+      <c r="I350" s="254"/>
+      <c r="J350" s="256"/>
+      <c r="K350" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L350" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M350" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="N350" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="O350" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="P350" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q350" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R350" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="S350" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T350" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="U350" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V350" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="W350" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="X350" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="AA350" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-001 (Must).</t>
+        </is>
+      </c>
+    </row>
+    <row r="351" ht="72.0" customHeight="1">
+      <c r="A351" s="253">
+        <v>19</v>
+      </c>
+      <c r="B351" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evaluation, Design &amp; Analysis</t>
+        </is>
+      </c>
+      <c r="C351" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D351" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evaluation, Design &amp; Analysis Details</t>
+        </is>
+      </c>
+      <c r="E351" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affected Personnel / Groups</t>
+        </is>
+      </c>
+      <c r="F351" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affected Personnel / Groups</t>
+        </is>
+      </c>
+      <c r="G351" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">People or groups to inform and train.</t>
+        </is>
+      </c>
+      <c r="H351" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+      <c r="I351" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tooltip: e.g. all operators at the terminal, maintenance contractor. Create Change Communication and Training tasks.</t>
+        </is>
+      </c>
+      <c r="J351" s="256"/>
+      <c r="K351" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L351" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M351" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="N351" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="O351" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="P351" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q351" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R351" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="S351" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T351" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="U351" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V351" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="W351" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="X351" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="AA351" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-016 (Must) / RULE-B3-10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="352" ht="28.8" customHeight="1">
+      <c r="A352" s="253">
+        <v>20</v>
+      </c>
+      <c r="B352" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow Up</t>
+        </is>
+      </c>
+      <c r="C352" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D352" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow-Up Details</t>
+        </is>
+      </c>
+      <c r="E352" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Field Verification (walk-around) Completed?</t>
+        </is>
+      </c>
+      <c r="F352" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Field Verification (walk-around) Completed?</t>
+        </is>
+      </c>
+      <c r="G352" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post-MoC field check.</t>
+        </is>
+      </c>
+      <c r="H352" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes/No</t>
+        </is>
+      </c>
+      <c r="I352" s="254"/>
+      <c r="J352" s="256"/>
+      <c r="K352" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L352" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M352" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="N352" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="O352" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P352" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q352" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R352" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="S352" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T352" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="U352" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V352" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="W352" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="X352" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="AA352" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-012 (Must).</t>
+        </is>
+      </c>
+    </row>
+    <row r="353" ht="28.8" customHeight="1">
+      <c r="A353" s="253">
+        <v>21</v>
+      </c>
+      <c r="B353" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow Up</t>
+        </is>
+      </c>
+      <c r="C353" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D353" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow-Up Details</t>
+        </is>
+      </c>
+      <c r="E353" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affected Personnel Interviewed / Communication Confirmed?</t>
+        </is>
+      </c>
+      <c r="F353" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Affected Personnel Interviewed / Communication Confirmed?</t>
+        </is>
+      </c>
+      <c r="G353" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post-MoC communication check.</t>
+        </is>
+      </c>
+      <c r="H353" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes/No</t>
+        </is>
+      </c>
+      <c r="I353" s="254"/>
+      <c r="J353" s="256"/>
+      <c r="K353" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L353" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M353" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="N353" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="O353" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P353" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q353" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R353" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="S353" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T353" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="U353" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V353" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="W353" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="X353" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="AA353" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-012 (Must).</t>
+        </is>
+      </c>
+    </row>
+    <row r="354" ht="28.8" customHeight="1">
+      <c r="A354" s="253">
+        <v>22</v>
+      </c>
+      <c r="B354" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow Up</t>
+        </is>
+      </c>
+      <c r="C354" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOC</t>
+        </is>
+      </c>
+      <c r="D354" s="255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Follow-Up Details</t>
+        </is>
+      </c>
+      <c r="E354" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Downstream &amp; Cumulative Impacts Reviewed?</t>
+        </is>
+      </c>
+      <c r="F354" s="257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Downstream &amp; Cumulative Impacts Reviewed?</t>
+        </is>
+      </c>
+      <c r="G354" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post-MoC impact review.</t>
+        </is>
+      </c>
+      <c r="H354" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes/No</t>
+        </is>
+      </c>
+      <c r="I354" s="254"/>
+      <c r="J354" s="256"/>
+      <c r="K354" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="L354" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="M354" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="N354" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="O354" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="P354" s="267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="Q354" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="R354" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="S354" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="T354" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="U354" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="V354" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="W354" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="X354" s="253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="AA354" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-012 (Must).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add internal MoC workshop questions and reword approval decisions
Questions list tags each open point with its source. Decision on
classification no longer framed as a blocker; BRD deviation entry
replaced by an open question on the number of approvers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018d6Sqji3PhM1w1Xd54RvCw
</commit_message>
<xml_diff>
--- a/docs/moc/Impala - Configuration Workbook - Management of Change v1.2 (Impala requirements DRAFT).xlsx
+++ b/docs/moc/Impala - Configuration Workbook - Management of Change v1.2 (Impala requirements DRAFT).xlsx
@@ -36626,7 +36626,7 @@
       </c>
       <c r="D10" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROPOSED (20-Oct): Minor = Local (TM), Moderate = Regional (HSEC + Ops), Major = Global (HSEC + Ops). Grade descriptors per type + 'Automatic Major' list (floating roof/deck landing, tank entry, SCE...). Pending sign-off by Global HSE (Stylianos). Procedure update + retraining required.</t>
+          <t xml:space="preserve">AGREED internally (20-Oct), per 'MOC Proposal.xlsx' (Sam): Minor = Local (TM), Moderate = Regional (HSEC + Ops), Major = Global (HSEC + Ops). Grade descriptors per type + 'Automatic Major' examples. Sam to circulate the updated matrix; Shaun to explain the rationale to Stylianos (internal alignment, not a configuration blocker). Procedure update + retraining required.</t>
         </is>
       </c>
       <c r="E10" s="52"/>
@@ -36826,17 +36826,17 @@
       </c>
       <c r="B20" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ratify deviations from approved BRD BO-61 v2.0 (B.3)</t>
+          <t xml:space="preserve">Minimum number of approvers per grade</t>
         </is>
       </c>
       <c r="C20" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala - Shaun Jones (MoC Process Owner)</t>
+          <t xml:space="preserve">Impala - Sam Robinson</t>
         </is>
       </c>
       <c r="D20" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">The 20-Oct design prevails but deviates from the approved BRD: (a) Level 0-5 scoring (FR-B3-006, RULE-B3-04) replaced by Type x Grade; (b) like-for-like exclusions not recorded in the system (FR-B3-002, Must) - rationale kept in the procedure; (c) Minor = single Terminal Manager approval vs RULE-B3-06 minimum of 2 approvers for Levels 0-3. Update Requirements Register BO61-203 and procedure CO-HS-GEN-PRO-002.</t>
+          <t xml:space="preserve">OPEN (internal workshop 21-Oct): 'MOC Proposal' defines the approval LEVEL per grade (Minor = Local - TM) but not the NUMBER of approvers. Current procedure/BRD: min. 2 approvers for lower levels, 3 for the highest. Confirm the rule to give Intelex. Note: Sam's design replaces Level 0-5 scoring and removes like-for-like from the module; BRD BO-61 to be updated accordingly (housekeeping).</t>
         </is>
       </c>
       <c r="E20" s="52"/>

</xml_diff>

<commit_message>
Add internal workshop questions workbook; put Replacement in Kind on hold
Replacement in Kind may be re-used as the simplified MOC switch, so it is
no longer flagged for removal in the configuration workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018d6Sqji3PhM1w1Xd54RvCw
</commit_message>
<xml_diff>
--- a/docs/moc/Impala - Configuration Workbook - Management of Change v1.2 (Impala requirements DRAFT).xlsx
+++ b/docs/moc/Impala - Configuration Workbook - Management of Change v1.2 (Impala requirements DRAFT).xlsx
@@ -30799,7 +30799,7 @@
       </c>
       <c r="N6" s="275" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - columns: Replacement in Kind removed; Type of Change + Grade of Change. Grouping by Status instead of Category [TBC].</t>
+          <t xml:space="preserve">M - columns: Replacement in Kind removed (unless re-used as 'Simplified MOC?' [TBC]); Type of Change + Grade of Change. Grouping by Status instead of Category [TBC].</t>
         </is>
       </c>
     </row>
@@ -36547,23 +36547,23 @@
       </c>
       <c r="E6" s="52"/>
     </row>
-    <row r="7" x14ac:dyDescent="0.55000000000000004" ht="28.8" customHeight="1">
+    <row r="7" x14ac:dyDescent="0.55000000000000004" ht="57.6" customHeight="1">
       <c r="A7" s="5">
         <v>3</v>
       </c>
       <c r="B7" s="215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Remove 'Replacement in Kind' (field and workflow path)</t>
+          <t xml:space="preserve">Replacement in Kind: remove or re-use as 'Simplified MOC' route</t>
         </is>
       </c>
       <c r="C7" s="215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala - Sam Robinson</t>
+          <t xml:space="preserve">Impala - Sam Robinson / Rodrigo Llamas</t>
         </is>
       </c>
       <c r="D7" s="215" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECIDED (Impala internal 20-Oct). Per Impala MoC procedure a like-for-like replacement is not a change, so it is out of MoC scope.</t>
+          <t xml:space="preserve">ON HOLD (internal workshop 21-Oct). 20-Oct: like-for-like is not a change per procedure, so the field as such is not needed. But its OOTB skip-path could be re-captioned (e.g. 'Simplified MOC?') to give the simplified route for organisational / IT changes without a new workflow. Decide: remove, or re-use (and define which stages it skips).</t>
         </is>
       </c>
       <c r="E7" s="52"/>
@@ -37103,7 +37103,7 @@
       </c>
       <c r="J68" s="239" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - Impala proposal (internal pre-design 20-Oct-2026, 'MOC Proposal.xlsx'). 6 stages instead of 7. Replacement in Kind path removed. The diagram above shows the OOTB workflow and must be redrawn by Intelex.</t>
+          <t xml:space="preserve">M - Impala proposal (internal pre-design 20-Oct-2026, 'MOC Proposal.xlsx'). 6 stages instead of 7. Replacement in Kind path ON HOLD: may be re-used as the 'Simplified MOC' route [TBC]. The diagram above shows the OOTB workflow and must be redrawn by Intelex.</t>
         </is>
       </c>
     </row>
@@ -41348,12 +41348,14 @@
       <c r="I16" s="187" t="s">
         <v>564</v>
       </c>
-      <c r="J16" s="187" t="s">
-        <v>565</v>
+      <c r="J16" s="254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[TBC] Remove, or re-caption as 'Simplified MOC?' re-using the OOTB skip path (organisational / IT changes).</t>
+        </is>
       </c>
       <c r="K16" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">R</t>
+          <t xml:space="preserve">M</t>
         </is>
       </c>
       <c r="L16" s="187" t="s">
@@ -41403,7 +41405,7 @@
       <c r="Z16" s="253"/>
       <c r="AA16" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Out of MoC scope per Impala procedure (like-for-like is not a change). Remove field and workflow path.</t>
+          <t xml:space="preserve">ON HOLD: like-for-like is out of MoC scope, but the field/path may become the simplified-MOC switch (decision 21-Oct).</t>
         </is>
       </c>
       <c r="AB16" s="61"/>

</xml_diff>

<commit_message>
Update MoC workbook and question list with internal session 2 (21-Oct)
Workflow and automatic sequential approvals confirmed; local approval
requires functional review plus TM; tasks kept (Action Plans optional);
task completion stage added; approval SLA 7 days; approval types no
longer re-captioned pending Intelex proposal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018d6Sqji3PhM1w1Xd54RvCw
</commit_message>
<xml_diff>
--- a/docs/moc/Impala - Configuration Workbook - Management of Change v1.2 (Impala requirements DRAFT).xlsx
+++ b/docs/moc/Impala - Configuration Workbook - Management of Change v1.2 (Impala requirements DRAFT).xlsx
@@ -6573,6 +6573,9 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="33" fillId="10" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -6596,9 +6599,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyAlignment="1" applyFill="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="10" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -28962,8 +28962,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DecisionsTasks" displayName="DecisionsTasks" ref="A4:E25" totalsRowCount="1" headerRowDxfId="1946" headerRowBorderDxfId="1945">
-  <autoFilter ref="A4:E24" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DecisionsTasks" displayName="DecisionsTasks" ref="A4:E30" totalsRowCount="1" headerRowDxfId="1946" headerRowBorderDxfId="1945">
+  <autoFilter ref="A4:E29" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" totalsRowLabel="Totals" dataDxfId="1944"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Task or Decision" totalsRowFunction="count" totalsRowDxfId="1943"/>
@@ -29471,8 +29471,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table5" displayName="Table5" ref="A5:E12" totalsRowCount="1" headerRowDxfId="1907" dataDxfId="1905" headerRowBorderDxfId="1906" dataCellStyle="20% - Accent1">
-  <autoFilter ref="A5:E11" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table5" displayName="Table5" ref="A5:E13" totalsRowCount="1" headerRowDxfId="1907" dataDxfId="1905" headerRowBorderDxfId="1906" dataCellStyle="20% - Accent1">
+  <autoFilter ref="A5:E12" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="Role Name" totalsRowLabel="Total" dataDxfId="1904" totalsRowDxfId="1903" dataCellStyle="20% - Accent1"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Description" dataDxfId="1902" totalsRowDxfId="1901" dataCellStyle="20% - Accent1"/>
@@ -30030,7 +30030,7 @@
       </c>
       <c r="E28" s="214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala requirements - DRAFT for Design Workshop (27-Oct-2026). Sources: ILX App Overview 19-Oct-2026, Impala internal pre-design 20-Oct-2026, 'MOC Proposal.xlsx' (priority), BRD BO-61 v2.0 B.3 (complementary), SOW v1.5. Changes flagged A/R/M, highlighted in yellow, rationale in 'Impala Notes' columns. Open points marked [TBC].</t>
+          <t xml:space="preserve">Impala requirements - DRAFT for Design Workshop (27-Oct-2026). Sources: ILX App Overview 19-Oct-2026, Impala internal pre-design sessions 20-Oct and 21-Oct-2026, 'MOC Proposal.xlsx' (priority), BRD BO-61 v2.0 B.3 (complementary), SOW v1.5. Changes flagged A/R/M, highlighted in yellow, rationale in 'Impala Notes' columns. Open points marked [TBC].</t>
         </is>
       </c>
       <c r="F28" s="214" t="inlineStr">
@@ -31561,7 +31561,7 @@
       </c>
       <c r="H14" s="250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approval object captions change (Local / Regional / Global) - permissions unchanged.</t>
+          <t xml:space="preserve">Approval types to be adapted (functional + level approvals) - permissions per type unchanged.</t>
         </is>
       </c>
     </row>
@@ -36467,7 +36467,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultColWidth="29.5234375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -36547,7 +36547,7 @@
       </c>
       <c r="E6" s="52"/>
     </row>
-    <row r="7" x14ac:dyDescent="0.55000000000000004" ht="57.6" customHeight="1">
+    <row r="7" x14ac:dyDescent="0.55000000000000004" ht="72.0" customHeight="1">
       <c r="A7" s="5">
         <v>3</v>
       </c>
@@ -36563,12 +36563,12 @@
       </c>
       <c r="D7" s="215" t="inlineStr">
         <is>
-          <t xml:space="preserve">ON HOLD (internal workshop 21-Oct). 20-Oct: like-for-like is not a change per procedure, so the field as such is not needed. But its OOTB skip-path could be re-captioned (e.g. 'Simplified MOC?') to give the simplified route for organisational / IT changes without a new workflow. Decide: remove, or re-use (and define which stages it skips).</t>
+          <t xml:space="preserve">STILL OPEN after 21-Oct (Sam: 'remove it or use it for a simplified workflow, come back to that'). 20-Oct: like-for-like is not a change per procedure, so the field as such is not needed. But its OOTB skip-path could be re-captioned (e.g. 'Simplified MOC?') to give the simplified route for organisational / IT changes without a new workflow. Decide: remove, or re-use (and define which stages it skips).</t>
         </is>
       </c>
       <c r="E7" s="52"/>
     </row>
-    <row r="8" x14ac:dyDescent="0.55000000000000004" ht="57.6" customHeight="1">
+    <row r="8" x14ac:dyDescent="0.55000000000000004" ht="72.0" customHeight="1">
       <c r="A8" s="5">
         <v>4</v>
       </c>
@@ -36584,12 +36584,12 @@
       </c>
       <c r="D8" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECIDED by Impala (20-Oct): remove Pre-Approval, merge Evaluation + Design &amp; Analysis, new Approval stage before Implementation, Emergency goes Initiation &gt; Approval. Intelex to confirm it fits SOW 'Moderate configuration' (minor modification of stages) - no Change Order expected by Impala.</t>
+          <t xml:space="preserve">CONFIRMED 21-Oct (Shaun: 'the workflow looks good'): remove Pre-Approval, merge Evaluation + Design &amp; Analysis, ONE main approval stage before Implementation (approve before construction/activity starts); pre-startup checks handled locally. Emergency route not discussed yet. Intelex to confirm it fits SOW 'Moderate configuration' (minor modification of stages) - no Change Order expected by Impala.</t>
         </is>
       </c>
       <c r="E8" s="52"/>
     </row>
-    <row r="9" x14ac:dyDescent="0.55000000000000004" ht="43.2" customHeight="1">
+    <row r="9" x14ac:dyDescent="0.55000000000000004" ht="57.6" customHeight="1">
       <c r="A9" s="5">
         <v>5</v>
       </c>
@@ -36605,12 +36605,12 @@
       </c>
       <c r="D9" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">REQUIRED: Terminal Manager approves first; Regional approvals only requested after Local is closed; Global only after Regional. OOTB approvals are not ordered. Intelex to propose solution (native ordering, sub-stages or action handler) and scope impact.</t>
+          <t xml:space="preserve">CONFIRMED 21-Oct: Major = Local &gt; Regional &gt; Global; as soon as the TM approves, the next level must be added and triggered AUTOMATICALLY (Sam: 'leave less down to human error'), not entered manually by the TM. OOTB approvals are not ordered. Intelex to propose solution (native ordering, sub-stages or action handler) and scope impact.</t>
         </is>
       </c>
       <c r="E9" s="52"/>
     </row>
-    <row r="10" x14ac:dyDescent="0.55000000000000004" ht="57.6" customHeight="1">
+    <row r="10" x14ac:dyDescent="0.55000000000000004" ht="100.8" customHeight="1">
       <c r="A10" s="5">
         <v>6</v>
       </c>
@@ -36626,12 +36626,12 @@
       </c>
       <c r="D10" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">AGREED internally (20-Oct), per 'MOC Proposal.xlsx' (Sam): Minor = Local (TM), Moderate = Regional (HSEC + Ops), Major = Global (HSEC + Ops). Grade descriptors per type + 'Automatic Major' examples. Sam to circulate the updated matrix; Shaun to explain the rationale to Stylianos (internal alignment, not a configuration blocker). Procedure update + retraining required.</t>
+          <t xml:space="preserve">21-Oct: Change Impact linked to the category (= type of change); matrix covers grade of change AND grade of hazard, so no scoring needed. Matrix OUT FOR TEAM REVIEW (check nothing previously Level 4 now comes out Minor). Per 'MOC Proposal.xlsx' (Sam): Minor = Local (TM), Moderate = Regional (HSEC + Ops), Major = Global (HSEC + Ops). Grade descriptors per type + 'Automatic Major' examples. Sam to circulate the updated matrix; Shaun to explain the rationale to Stylianos (internal alignment, not a configuration blocker). Procedure update + retraining required.</t>
         </is>
       </c>
       <c r="E10" s="52"/>
     </row>
-    <row r="11" x14ac:dyDescent="0.55000000000000004" ht="43.2" customHeight="1">
+    <row r="11" x14ac:dyDescent="0.55000000000000004" ht="57.6" customHeight="1">
       <c r="A11" s="5">
         <v>7</v>
       </c>
@@ -36647,39 +36647,39 @@
       </c>
       <c r="D11" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checklist 'Evaluation, D&amp;A Checklist' loaded as screening questions (Excel import). Part 1 at top location, Part 2 at Liquids segment, Part 3 at Dry segment. Open: reduce question set by Grade (Minor short list, Major full) [TBC]. Location-specific checklists = Phase 2.</t>
+          <t xml:space="preserve">Checklist 'Evaluation, D&amp;A Checklist' loaded as screening questions (Excel import). Part 1 at top location, Part 2 at Liquids segment, Part 3 at Dry segment (triggered by location - confirmed 21-Oct). List under team review. OPEN: same checklist for all changes, or questions shown only for certain types of change [TBC]. Location-specific checklists = Phase 2.</t>
         </is>
       </c>
       <c r="E11" s="52"/>
     </row>
-    <row r="12" x14ac:dyDescent="0.55000000000000004" ht="43.2" customHeight="1">
+    <row r="12" x14ac:dyDescent="0.55000000000000004" ht="57.6" customHeight="1">
       <c r="A12" s="5">
         <v>8</v>
       </c>
       <c r="B12" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Link Action Plans to the MOC</t>
+          <t xml:space="preserve">MOC Tasks vs Action Plans</t>
         </is>
       </c>
       <c r="C12" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intelex - Ian</t>
+          <t xml:space="preserve">Impala - Shaun Jones / Intelex - Ian</t>
         </is>
       </c>
       <c r="D12" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">REQUIRED: actions arising from the MOC (permits, licences, site checks) raised as Action Plans with traceability back to the MOC No. (grid on MOC). Intelex to confirm feasibility (Action Plans in Phase 1 scope).</t>
+          <t xml:space="preserve">21-Oct: keep MOC TASKS as the MOC actions (Shaun: tasks are part of the MOC; if overdue, the MOC is overdue). Sam would prefer Action Plans (single overdue-actions reporting) but is 'happy either way'; Alonso: replacing tasks with Action Plans is probably not a minor change. Ask Intelex only for effort of an Action Plans link (nice-to-have).</t>
         </is>
       </c>
       <c r="E12" s="52"/>
     </row>
-    <row r="13" x14ac:dyDescent="0.55000000000000004" ht="43.2" customHeight="1">
+    <row r="13" x14ac:dyDescent="0.55000000000000004" ht="57.6" customHeight="1">
       <c r="A13" s="5">
         <v>9</v>
       </c>
       <c r="B13" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Simplified MOC workflow (organisational / IT changes)</t>
+          <t xml:space="preserve">Task completion stage (pre-startup vs post-startup)</t>
         </is>
       </c>
       <c r="C13" s="216" t="inlineStr">
@@ -36689,39 +36689,39 @@
       </c>
       <c r="D13" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPEN: Intelex to confirm whether the simplified/'Change Request' workflow seen in the demo site is in SOW. Impala priority: finalise the full MOC first; Emergency kept minimal (low volume).</t>
+          <t xml:space="preserve">REQUIRED 21-Oct (Khesar / Sam): OOTB a stage cannot be submitted with open tasks, but some tasks identified in Evaluation are only due later (e.g. P&amp;ID update post-change). Add on each MOC Task a 'Complete before stage' field (Implementation / Start Up / Follow Up); the stage gate checks only tasks due for that stage. Covers BRD FR-B3-032.</t>
         </is>
       </c>
       <c r="E13" s="52"/>
     </row>
-    <row r="14" x14ac:dyDescent="0.55000000000000004" ht="43.2" customHeight="1">
+    <row r="14" x14ac:dyDescent="0.55000000000000004" ht="57.6" customHeight="1">
       <c r="A14" s="5">
         <v>10</v>
       </c>
       <c r="B14" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage gating rules</t>
+          <t xml:space="preserve">Local (Minor) approval: no single-person MOC</t>
         </is>
       </c>
       <c r="C14" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala - Sam Robinson</t>
+          <t xml:space="preserve">Impala - Shaun Jones</t>
         </is>
       </c>
       <c r="D14" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">REQUIRED: OOTB nothing forces tasks/approvals per stage. Proposed: all screening questions answered + stage tasks closed before Approval; at least one approval (Local) and all approvals closed before Implementation.</t>
+          <t xml:space="preserve">21-Oct (Shaun): a MOC must never be raised, completed and approved by one person (seen in Sphera, e.g. Rotterdam). Local approval = functional review (Operations / Maintenance, other specialists) + Terminal Manager final sign-off (Khesar). Automatic where possible; specialist input (e.g. electrical) may be proceduralised (Sam).</t>
         </is>
       </c>
       <c r="E14" s="52"/>
     </row>
-    <row r="15" ht="28.8" customHeight="1">
+    <row r="15" ht="72.0" customHeight="1">
       <c r="A15" s="217">
         <v>11</v>
       </c>
       <c r="B15" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approvals generated only after evaluation is complete</t>
+          <t xml:space="preserve">Approval types list</t>
         </is>
       </c>
       <c r="C15" s="216" t="inlineStr">
@@ -36731,28 +36731,28 @@
       </c>
       <c r="D15" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Resolved by design: approvals auto-generate on entry to the Approval stage (after the checklist). Intelex to confirm generation timing.</t>
+          <t xml:space="preserve">21-Oct: OOTB types (Engineering, Environmental, Safety, Risk Mgmt, Financial, Start Up) kept so users can add functional approvals; 'Operations' missing (Khesar); list to be adapted to the business. Needed: functional types (Operations, Maintenance, Engineering, Safety, Environmental) + level approvals (TM, Regional HSEC/Ops, Global HSEC/Ops). Intelex to propose (re-caption existing objects vs new).</t>
         </is>
       </c>
       <c r="E15" s="52"/>
     </row>
-    <row r="16" ht="28.8" customHeight="1">
+    <row r="16" ht="57.6" customHeight="1">
       <c r="A16" s="217">
         <v>12</v>
       </c>
       <c r="B16" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">External parties (contractors) in tasks/approvals</t>
+          <t xml:space="preserve">Manual MOC form retired - digital only</t>
         </is>
       </c>
       <c r="C16" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala - Alonso Maranon Barrios</t>
+          <t xml:space="preserve">Impala - Shaun Jones</t>
         </is>
       </c>
       <c r="D16" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECIDED: no Intelex access for externals; internal owner of the task collects and uploads evidence. Public Forms are not in SOW.</t>
+          <t xml:space="preserve">DECIDED 21-Oct: no paper/Word MOC form (it only existed because of the Sphera approver limit). Supporting documents (JSA/risk assessment, method statements, procedures, P&amp;IDs, design documents) attached in Intelex; instruction text under Attachments listing expected documents (Khesar).</t>
         </is>
       </c>
       <c r="E16" s="52"/>
@@ -36763,101 +36763,101 @@
       </c>
       <c r="B17" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Security groups and location roles population</t>
+          <t xml:space="preserve">Per-stage requirements map</t>
         </is>
       </c>
       <c r="C17" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala - Rodrigo Llamas</t>
+          <t xml:space="preserve">Impala - Sam Robinson</t>
         </is>
       </c>
       <c r="D17" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Users/groups via Workday (EDIS) feed; location roles (MOC Coordinator, Terminal Manager, Regional/Global approvers) nominated per terminal/region. Local variations handled by role assignment, not by workflow.</t>
+          <t xml:space="preserve">ACTION 21-Oct (Shaun): map per stage what we ask, which documents we expect/mandate and where we approve. Sam to update his workbook (EOD 21-Oct); Rodrigo to transfer to this workbook. Also: Follow Up questions from the MOC audit form (Sam).</t>
         </is>
       </c>
       <c r="E17" s="52"/>
     </row>
-    <row r="18" ht="14.4" customHeight="1">
+    <row r="18" ht="43.2" customHeight="1">
       <c r="A18" s="217">
         <v>14</v>
       </c>
       <c r="B18" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stage due dates, reminders and escalations</t>
+          <t xml:space="preserve">Simplified MOC workflow (organisational / IT changes)</t>
         </is>
       </c>
       <c r="C18" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala - Shaun Jones</t>
+          <t xml:space="preserve">Intelex - Ian</t>
         </is>
       </c>
       <c r="D18" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPEN: confirm SLAs per stage and the escalation ladder proposed in 'Notification Schedules'.</t>
+          <t xml:space="preserve">OPEN: Intelex to confirm whether the simplified/'Change Request' workflow seen in the demo site is in SOW. Impala priority: finalise the full MOC first; Emergency kept minimal (low volume).</t>
         </is>
       </c>
       <c r="E18" s="52"/>
     </row>
-    <row r="19" ht="28.8" customHeight="1">
+    <row r="19" ht="57.6" customHeight="1">
       <c r="A19" s="217">
         <v>15</v>
       </c>
       <c r="B19" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Translations of custom configuration (ES)</t>
+          <t xml:space="preserve">Stage gating rules</t>
         </is>
       </c>
       <c r="C19" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala - Rodrigo Llamas</t>
+          <t xml:space="preserve">Impala - Sam Robinson</t>
         </is>
       </c>
       <c r="D19" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Per SOW Impala translates custom captions, tooltips, instructions and e-mails (OOTB ES/FR/PT/ZH provided).</t>
+          <t xml:space="preserve">CONFIRMED 21-Oct: in the demo Sam reached Start Up without answering the stage questions - must be impossible. OOTB nothing forces tasks/approvals per stage. Proposed: all screening questions answered + stage tasks closed before Approval; at least one approval (Local) and all approvals closed before Implementation.</t>
         </is>
       </c>
       <c r="E19" s="52"/>
     </row>
-    <row r="20" ht="72.0" customHeight="1">
+    <row r="20" ht="28.8" customHeight="1">
       <c r="A20" s="217">
         <v>16</v>
       </c>
       <c r="B20" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Minimum number of approvers per grade</t>
+          <t xml:space="preserve">Approvals generated only after evaluation is complete</t>
         </is>
       </c>
       <c r="C20" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala - Sam Robinson</t>
+          <t xml:space="preserve">Intelex - Ian</t>
         </is>
       </c>
       <c r="D20" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPEN (internal workshop 21-Oct): 'MOC Proposal' defines the approval LEVEL per grade (Minor = Local - TM) but not the NUMBER of approvers. Current procedure/BRD: min. 2 approvers for lower levels, 3 for the highest. Confirm the rule to give Intelex. Note: Sam's design replaces Level 0-5 scoring and removes like-for-like from the module; BRD BO-61 to be updated accordingly (housekeeping).</t>
+          <t xml:space="preserve">Resolved by design: approvals auto-generate on entry to the Approval stage (after the checklist). Intelex to confirm generation timing.</t>
         </is>
       </c>
       <c r="E20" s="52"/>
     </row>
-    <row r="21" ht="43.2" customHeight="1">
+    <row r="21" ht="28.8" customHeight="1">
       <c r="A21" s="217">
         <v>17</v>
       </c>
       <c r="B21" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Return for revision vs formal rejection</t>
+          <t xml:space="preserve">External parties (contractors) in tasks/approvals</t>
         </is>
       </c>
       <c r="C21" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intelex - Ian</t>
+          <t xml:space="preserve">Impala - Alonso Maranon Barrios</t>
         </is>
       </c>
       <c r="D21" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">BRD FR-B3-035 (Must): Roll Back from Approval = return for revision, closed approvals are KEPT; formal rejection resets the approval chain (RULE-B3-07). Intelex to confirm OOTB behaviour of approvals on Roll Back.</t>
+          <t xml:space="preserve">DECIDED: no Intelex access for externals; internal owner of the task collects and uploads evidence. Public Forms are not in SOW.</t>
         </is>
       </c>
       <c r="E21" s="52"/>
@@ -36868,17 +36868,17 @@
       </c>
       <c r="B22" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emergency MOC regularisation</t>
+          <t xml:space="preserve">Security groups and location roles population</t>
         </is>
       </c>
       <c r="C22" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala - Shaun Jones</t>
+          <t xml:space="preserve">Impala - Rodrigo Llamas</t>
         </is>
       </c>
       <c r="D22" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">BRD RULE-B3-14: single senior approval, immediate execution, full dossier (checklist, tasks) completed retrospectively within [TBC] days; record flagged 'pending regularisation' and reported overdue; cannot be closed until regularised (AH17).</t>
+          <t xml:space="preserve">Users/groups via Workday (EDIS) feed; location roles (MOC Coordinator, Terminal Manager, Regional/Global approvers) nominated per terminal/region. Local variations handled by role assignment, not by workflow.</t>
         </is>
       </c>
       <c r="E22" s="52"/>
@@ -36889,51 +36889,156 @@
       </c>
       <c r="B23" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temporary change extensions</t>
+          <t xml:space="preserve">Stage due dates, reminders and escalations</t>
         </is>
       </c>
       <c r="C23" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impala - Sam Robinson</t>
+          <t xml:space="preserve">Impala - Shaun Jones</t>
         </is>
       </c>
       <c r="D23" s="216" t="inlineStr">
         <is>
-          <t xml:space="preserve">BRD RULE-B3-08 / FR-B3-014: review date, max 3 extensions each with rationale and re-approval at the MOC grade (ad hoc approval); conversion to permanent = new MOC linked through Related MOCs.</t>
+          <t xml:space="preserve">21-Oct (Sam): Evaluation/Design &amp; Analysis cannot have a fixed SLA (project size varies wildly); only the Approval stage gets one: approvals within 7 days. Escalation ladder for tasks = BA proposal, to be confirmed.</t>
         </is>
       </c>
       <c r="E23" s="52"/>
     </row>
-    <row r="24" ht="43.2" customHeight="1">
+    <row r="24" ht="28.8" customHeight="1">
       <c r="A24" s="217">
         <v>20</v>
       </c>
       <c r="B24" s="216" t="inlineStr">
         <is>
+          <t xml:space="preserve">Translations of custom configuration (ES)</t>
+        </is>
+      </c>
+      <c r="C24" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Impala - Rodrigo Llamas</t>
+        </is>
+      </c>
+      <c r="D24" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Per SOW Impala translates custom captions, tooltips, instructions and e-mails (OOTB ES/FR/PT/ZH provided).</t>
+        </is>
+      </c>
+      <c r="E24" s="52"/>
+    </row>
+    <row r="25" ht="43.2" customHeight="1">
+      <c r="A25" s="217">
+        <v>21</v>
+      </c>
+      <c r="B25" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minimum number of approvers per grade</t>
+        </is>
+      </c>
+      <c r="C25" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Impala - Sam Robinson</t>
+        </is>
+      </c>
+      <c r="D25" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PARTLY ANSWERED 21-Oct: Local = at least one functional reviewer (Ops/Maintenance) + TM (so &gt;= 2, in line with BRD). Regional and Global = HSEC + Operations. Exact rule per level to be written in Sam's per-stage map. BRD BO-61 to be updated for Level 0-5 scoring (housekeeping).</t>
+        </is>
+      </c>
+      <c r="E25" s="52"/>
+    </row>
+    <row r="26" ht="43.2" customHeight="1">
+      <c r="A26" s="217">
+        <v>22</v>
+      </c>
+      <c r="B26" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Return for revision vs formal rejection</t>
+        </is>
+      </c>
+      <c r="C26" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intelex - Ian</t>
+        </is>
+      </c>
+      <c r="D26" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD FR-B3-035 (Must): Roll Back from Approval = return for revision, closed approvals are KEPT; formal rejection resets the approval chain (RULE-B3-07). Intelex to confirm OOTB behaviour of approvals on Roll Back.</t>
+        </is>
+      </c>
+      <c r="E26" s="52"/>
+    </row>
+    <row r="27" ht="43.2" customHeight="1">
+      <c r="A27" s="217">
+        <v>23</v>
+      </c>
+      <c r="B27" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Emergency MOC regularisation</t>
+        </is>
+      </c>
+      <c r="C27" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Impala - Shaun Jones</t>
+        </is>
+      </c>
+      <c r="D27" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD RULE-B3-14: single senior approval, immediate execution, full dossier (checklist, tasks) completed retrospectively within [TBC] days; record flagged 'pending regularisation' and reported overdue; cannot be closed until regularised (AH17).</t>
+        </is>
+      </c>
+      <c r="E27" s="52"/>
+    </row>
+    <row r="28" ht="43.2" customHeight="1">
+      <c r="A28" s="217">
+        <v>24</v>
+      </c>
+      <c r="B28" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temporary change extensions</t>
+        </is>
+      </c>
+      <c r="C28" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Impala - Sam Robinson</t>
+        </is>
+      </c>
+      <c r="D28" s="216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BRD RULE-B3-08 / FR-B3-014: review date, max 3 extensions each with rationale and re-approval at the MOC grade (ad hoc approval); conversion to permanent = new MOC linked through Related MOCs (Related MOCs kept 21-Oct for traceability, e.g. phased tank works).</t>
+        </is>
+      </c>
+      <c r="E28" s="52"/>
+    </row>
+    <row r="29" ht="43.2" customHeight="1">
+      <c r="A29" s="217">
+        <v>25</v>
+      </c>
+      <c r="B29" s="216" t="inlineStr">
+        <is>
           <t xml:space="preserve">MoC KPIs and leadership reporting</t>
         </is>
       </c>
-      <c r="C24" s="216" t="inlineStr">
+      <c r="C29" s="216" t="inlineStr">
         <is>
           <t xml:space="preserve">Impala - Rodrigo Llamas</t>
         </is>
       </c>
-      <c r="D24" s="216" t="inlineStr">
+      <c r="D29" s="216" t="inlineStr">
         <is>
           <t xml:space="preserve">BRD FR-B3-019 / FR-B3-033: monthly YTD permanent/temporary MOCs, open MOCs, overdue temporary MOCs, MoC-related incidents, open MoC actions + leading indicators. To be built as reports/dashboards (reporting phase), fields already captured in this workbook.</t>
         </is>
       </c>
-      <c r="E24" s="52"/>
-    </row>
-    <row r="25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" t="s">
+      <c r="E29" s="52"/>
+    </row>
+    <row r="30" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" t="s">
         <v>77</v>
       </c>
-      <c r="B25" s="29">
+      <c r="B30" s="29">
         <f>SUBTOTAL(103,DecisionsTasks[Task or Decision])</f>
         <v>2</v>
       </c>
-      <c r="E25" s="29">
+      <c r="E30" s="29">
         <f>SUBTOTAL(103,DecisionsTasks[Date Complete])</f>
         <v>0</v>
       </c>
@@ -37098,7 +37203,7 @@
         <is>
           <t xml:space="preserve">Recipient(s): Change Requester, MOC Coordinator (Role)
 N11 to Terminal Manager + Regional HSEC if Emergency = Yes.
-Prior to submit: Change Description, Type of Change, Grade of Change, Grade Justification mandatory; Emergency Justification if Emergency = Yes; Change Expiry if Temporary = Yes.</t>
+Prior to submit: Change Description, Type of Change, Grade of Change, Reason for Change &amp; Technical Basis mandatory; Emergency Justification if Emergency = Yes; Change Expiry if Temporary = Yes.</t>
         </is>
       </c>
       <c r="J68" s="239" t="inlineStr">
@@ -37107,7 +37212,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="57.6" x14ac:dyDescent="0.55000000000000004" customHeight="1">
+    <row r="69" ht="72.0" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A69" s="133">
         <v>2</v>
       </c>
@@ -37126,7 +37231,7 @@
       </c>
       <c r="E69" s="220" t="inlineStr">
         <is>
-          <t xml:space="preserve">[TBC] e.g. 30 days from stage entry</t>
+          <t xml:space="preserve">N/A (project dependent - 21-Oct)</t>
         </is>
       </c>
       <c r="F69" s="14" t="s">
@@ -37144,7 +37249,7 @@
         <is>
           <t xml:space="preserve">Recipient(s): Change Requester
 Replaces OOTB Pre-Approval, Evaluation and Design &amp; Analysis stages.
-Prior to transitioning: all screening questions answered and all tasks of this stage closed.</t>
+Prior to transitioning: all screening questions and stage questions answered, design documents attached, and tasks whose 'Complete before stage' = Approval closed (tasks due later stay open).</t>
         </is>
       </c>
       <c r="J69" s="239" t="inlineStr">
@@ -37193,7 +37298,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="187.2" x14ac:dyDescent="0.55000000000000004" customHeight="1">
+    <row r="72" ht="201.6" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A72" s="136">
         <v>3</v>
       </c>
@@ -37212,7 +37317,7 @@
       </c>
       <c r="E72" s="226" t="inlineStr">
         <is>
-          <t xml:space="preserve">[TBC] e.g. 14 days from stage entry</t>
+          <t xml:space="preserve">7 days from stage entry (21-Oct)</t>
         </is>
       </c>
       <c r="F72" s="16" t="s">
@@ -37232,10 +37337,10 @@
         <is>
           <t xml:space="preserve">Recipient(s): Change Requester
 Approvals auto-generated on stage entry by Grade of Change:
-- Minor: Local (Terminal Manager)
+- Minor: Local = functional review (Operations / Maintenance) + Terminal Manager final sign-off
 - Moderate: Local &gt; Regional HSEC + Regional Operations
-- Major: Local &gt; Regional &gt; Global HSEC + Global Operations [TBC Regional step for Major]
-Approvals are SEQUENTIAL: next level requested only when the previous level is closed (Intelex to confirm solution).
+- Major: Local &gt; Regional &gt; Global HSEC + Global Operations (confirmed 21-Oct)
+Approvals are SEQUENTIAL and AUTOMATIC: when the TM approves, the next level is added and triggered by the system (Intelex to confirm solution). The single main approval happens here, before construction/activity starts.
 Ad hoc approvers can be added by the MOC Coordinator.
 Prior to transitioning: at least one approval exists and all approvals are closed (accepted).
 Roll Back = return for revision, closed approvals are kept; a formal rejection resets the chain (BRD FR-B3-035) [Intelex to confirm].</t>
@@ -37324,8 +37429,8 @@
       <c r="I75" s="223" t="inlineStr">
         <is>
           <t xml:space="preserve">Recipient(s): Change Requester
-Prior to transitioning to next stage, all tasks have to be completed.
-Tasks of this stage = pre-startup actions (incl. PSSR where required by Type/Grade): Start Up is blocked until they are closed (BRD FR-B3-028 / FR-B3-032). Post-startup actions are created in Follow Up.</t>
+Prior to transitioning: tasks with 'Complete before stage' = Start Up (pre-startup actions, PSSR) closed; Implementation questions answered. Post-startup tasks (e.g. P&amp;ID update) stay open until Follow Up (BRD FR-B3-028 / FR-B3-032).
+Optional local pre-startup approval [TBC] - main approval already given.</t>
         </is>
       </c>
     </row>
@@ -37924,7 +38029,7 @@
       </c>
       <c r="B4" s="241" t="inlineStr">
         <is>
-          <t xml:space="preserve">MOC Task / MOC Approval (reminders to Person Responsible)</t>
+          <t xml:space="preserve">MOC Approval (due 7 days after request - 21-Oct) and MOC Task (BA proposal [TBC])</t>
         </is>
       </c>
     </row>
@@ -37947,7 +38052,7 @@
     </row>
     <row r="6" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="242">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" s="242" t="inlineStr">
         <is>
@@ -37956,12 +38061,12 @@
       </c>
       <c r="C6" s="243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Person Responsible</t>
+          <t xml:space="preserve">Person Responsible (approver / task owner)</t>
         </is>
       </c>
       <c r="D6" s="242" t="inlineStr">
         <is>
-          <t xml:space="preserve">N13 / N14</t>
+          <t xml:space="preserve">N14 / N13</t>
         </is>
       </c>
       <c r="E6" s="244" t="inlineStr">
@@ -37986,7 +38091,7 @@
       </c>
       <c r="D7" s="245" t="inlineStr">
         <is>
-          <t xml:space="preserve">N13 / N14</t>
+          <t xml:space="preserve">N14 / N13</t>
         </is>
       </c>
       <c r="E7" s="244" t="inlineStr">
@@ -37997,7 +38102,7 @@
     </row>
     <row r="8" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="242">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B8" s="242" t="inlineStr">
         <is>
@@ -38011,18 +38116,18 @@
       </c>
       <c r="D8" s="242" t="inlineStr">
         <is>
-          <t xml:space="preserve">N13 / N14</t>
+          <t xml:space="preserve">N14 / N13</t>
         </is>
       </c>
       <c r="E8" s="244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every 7 days until closed</t>
+          <t xml:space="preserve">Every 3 days until closed [TBC]</t>
         </is>
       </c>
     </row>
     <row r="9" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="245">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B9" s="245" t="inlineStr">
         <is>
@@ -38036,7 +38141,7 @@
       </c>
       <c r="D9" s="245" t="inlineStr">
         <is>
-          <t xml:space="preserve">N13 / N14</t>
+          <t xml:space="preserve">N14 / N13</t>
         </is>
       </c>
       <c r="E9" s="244" t="inlineStr">
@@ -38872,76 +38977,76 @@
     <row r="8" s="29" customFormat="1" x14ac:dyDescent="0.55000000000000004" ht="43.2" customHeight="1">
       <c r="A8" s="250" t="inlineStr">
         <is>
+          <t xml:space="preserve">Terminal Functional Reviewer (Operations / Maintenance)</t>
+        </is>
+      </c>
+      <c r="B8" s="251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Local functional review before the Terminal Manager sign-off, so no MOC is raised and approved by one person (21-Oct). Specialists (e.g. electrical) added ad hoc.</t>
+        </is>
+      </c>
+      <c r="C8" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Group</t>
+        </is>
+      </c>
+      <c r="D8" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="E8" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workflow Task</t>
+        </is>
+      </c>
+      <c r="F8" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A - 21-Oct (Shaun, Khesar). Automatic local approval step [TBC with Intelex].</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" x14ac:dyDescent="0.55000000000000004" ht="43.2" customHeight="1">
+      <c r="A9" s="250" t="inlineStr">
+        <is>
           <t xml:space="preserve">Regional HSEC Manager</t>
         </is>
       </c>
-      <c r="B8" s="251" t="inlineStr">
+      <c r="B9" s="251" t="inlineStr">
         <is>
           <t xml:space="preserve">Regional approver for Moderate and Major changes. Notified of Emergency MOCs.</t>
         </is>
       </c>
-      <c r="C8" s="250" t="inlineStr">
+      <c r="C9" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">Individual</t>
         </is>
       </c>
-      <c r="D8" s="250" t="inlineStr">
+      <c r="D9" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="E8" s="250" t="inlineStr">
+      <c r="E9" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">Workflow Task, Location-Based Notification</t>
         </is>
       </c>
-      <c r="F8" s="250" t="inlineStr">
+      <c r="F9" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">A - Regional approval level. Local variations (e.g. a different approver for a region) handled by role assignment, not by workflow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" x14ac:dyDescent="0.55000000000000004" ht="28.8" customHeight="1">
-      <c r="A9" s="250" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Regional Operations Manager</t>
-        </is>
-      </c>
-      <c r="B9" s="251" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Regional approver for Moderate and Major changes.</t>
-        </is>
-      </c>
-      <c r="C9" s="250" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Individual</t>
-        </is>
-      </c>
-      <c r="D9" s="250" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Y</t>
-        </is>
-      </c>
-      <c r="E9" s="250" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Workflow Task</t>
-        </is>
-      </c>
-      <c r="F9" s="250" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A - Regional approval level. BRD FR-B3-007: ROM / Country Operations Manager.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28.8" customHeight="1">
       <c r="A10" s="250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Global HSEC</t>
+          <t xml:space="preserve">Regional Operations Manager</t>
         </is>
       </c>
       <c r="B10" s="251" t="inlineStr">
         <is>
-          <t xml:space="preserve">Global approver for Major changes.</t>
+          <t xml:space="preserve">Regional approver for Moderate and Major changes.</t>
         </is>
       </c>
       <c r="C10" s="250" t="inlineStr">
@@ -38961,60 +39066,85 @@
       </c>
       <c r="F10" s="250" t="inlineStr">
         <is>
-          <t xml:space="preserve">A - Global approval level (assigned at top location). BRD FR-B3-007: Head of HSEQ.</t>
+          <t xml:space="preserve">A - Regional approval level. BRD FR-B3-007: ROM / Country Operations Manager.</t>
         </is>
       </c>
     </row>
     <row r="11" x14ac:dyDescent="0.55000000000000004" ht="28.8" customHeight="1">
       <c r="A11" s="250" t="inlineStr">
         <is>
+          <t xml:space="preserve">Global HSEC</t>
+        </is>
+      </c>
+      <c r="B11" s="251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Global approver for Major changes.</t>
+        </is>
+      </c>
+      <c r="C11" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Individual</t>
+        </is>
+      </c>
+      <c r="D11" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="E11" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Workflow Task</t>
+        </is>
+      </c>
+      <c r="F11" s="250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A - Global approval level (assigned at top location). BRD FR-B3-007: Head of HSEQ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" x14ac:dyDescent="0.55000000000000004" ht="28.8" customHeight="1">
+      <c r="A12" s="250" t="inlineStr">
+        <is>
           <t xml:space="preserve">Global Operations</t>
         </is>
       </c>
-      <c r="B11" s="251" t="inlineStr">
+      <c r="B12" s="251" t="inlineStr">
         <is>
           <t xml:space="preserve">Global approver for Major changes.</t>
         </is>
       </c>
-      <c r="C11" s="250" t="inlineStr">
+      <c r="C12" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">Individual</t>
         </is>
       </c>
-      <c r="D11" s="250" t="inlineStr">
+      <c r="D12" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="E11" s="250" t="inlineStr">
+      <c r="E12" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">Workflow Task</t>
         </is>
       </c>
-      <c r="F11" s="250" t="inlineStr">
+      <c r="F12" s="250" t="inlineStr">
         <is>
           <t xml:space="preserve">A - Global approval level (assigned at top location). BRD FR-B3-007: COO.</t>
         </is>
       </c>
     </row>
-    <row r="12" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="1" t="s">
+    <row r="13" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="53">
+      <c r="B13" s="1"/>
+      <c r="C13" s="53">
         <f>SUBTOTAL(103,Table5[Individual / Group])</f>
         <v>1</v>
       </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
     </row>
     <row r="14" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="3"/>
@@ -39347,7 +39477,7 @@
       </c>
       <c r="N47" s="245" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - caption: 'Local Approval (Terminal Manager)'</t>
+          <t xml:space="preserve">Keep as functional approval (21-Oct). See decision 'Approval types list'.</t>
         </is>
       </c>
     </row>
@@ -39393,7 +39523,7 @@
       </c>
       <c r="N48" s="245" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - caption: 'Regional Operations Approval'</t>
+          <t xml:space="preserve">Keep as functional approval (21-Oct).</t>
         </is>
       </c>
     </row>
@@ -39439,7 +39569,7 @@
       </c>
       <c r="N49" s="245" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - caption: 'Global Operations Approval'</t>
+          <t xml:space="preserve">[TBC] re-use for a missing type (e.g. Operations / Maintenance / level approval) - Intelex to propose.</t>
         </is>
       </c>
     </row>
@@ -39971,7 +40101,7 @@
       </c>
       <c r="N62" s="245" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - caption: 'Global HSEC Approval'</t>
+          <t xml:space="preserve">[TBC] re-use for a missing type - Intelex to propose.</t>
         </is>
       </c>
     </row>
@@ -40017,7 +40147,7 @@
       </c>
       <c r="N63" s="245" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - caption: 'Regional HSEC Approval'</t>
+          <t xml:space="preserve">Keep as functional approval (21-Oct).</t>
         </is>
       </c>
     </row>
@@ -40063,7 +40193,7 @@
       </c>
       <c r="N64" s="245" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - caption: 'Additional Approval (ad hoc)'</t>
+          <t xml:space="preserve">[TBC] re-use for a missing type - Intelex to propose.</t>
         </is>
       </c>
     </row>
@@ -41755,12 +41885,12 @@
       <c r="Z20" s="253"/>
       <c r="AA20" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not used: Grade of Change is the single criticality driver.</t>
+          <t xml:space="preserve">Not used: Grade of Change is the single criticality driver (Sam 21-Oct: not sure Priority drives anything).</t>
         </is>
       </c>
       <c r="AB20" s="61"/>
     </row>
-    <row r="21" s="59" customFormat="1" ht="57.6" x14ac:dyDescent="0.55000000000000004" customHeight="1">
+    <row r="21" s="59" customFormat="1" ht="72.0" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A21" s="188">
         <v>17</v>
       </c>
@@ -41775,12 +41905,12 @@
       </c>
       <c r="E21" s="257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grade Justification</t>
+          <t xml:space="preserve">Reason for Change &amp; Technical Basis</t>
         </is>
       </c>
       <c r="F21" s="257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grade Justification</t>
+          <t xml:space="preserve">Reason for Change &amp; Technical Basis</t>
         </is>
       </c>
       <c r="G21" s="187" t="s">
@@ -41791,12 +41921,12 @@
       </c>
       <c r="I21" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tooltip: Explain why the selected grade applies (reference the descriptor or the Automatic Major list).</t>
+          <t xml:space="preserve">Tooltip: Why the change is needed, technical basis, scope, current situation and what approvers should look out for.</t>
         </is>
       </c>
       <c r="J21" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text. Mandatory.</t>
+          <t xml:space="preserve">Text (multi-line, no length limit). Mandatory.</t>
         </is>
       </c>
       <c r="K21" s="254" t="inlineStr">
@@ -41851,7 +41981,7 @@
       <c r="Z21" s="253"/>
       <c r="AA21" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Re-purposed Priority Explanation.</t>
+          <t xml:space="preserve">21-Oct (Khesar, agreed by Sam): Priority Explanation re-worded as reason / technical basis - gives approvers context. Covers BRD FR-B3-001.</t>
         </is>
       </c>
       <c r="AB21" s="61"/>
@@ -42266,7 +42396,7 @@
       <c r="Z26" s="253"/>
       <c r="AA26" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approvals now controlled in the Approval stage.</t>
+          <t xml:space="preserve">CONFIRMED 21-Oct (Shaun: 'it's the point of the approval'). Approvals controlled in the Approval stage.</t>
         </is>
       </c>
     </row>
@@ -42440,7 +42570,7 @@
       <c r="Z28" s="253"/>
       <c r="AA28" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moved to combined stage.</t>
+          <t xml:space="preserve">Moved to combined stage. 21-Oct: keep 'Alternatives Considered' (important).</t>
         </is>
       </c>
     </row>
@@ -42701,7 +42831,7 @@
       <c r="Z31" s="253"/>
       <c r="AA31" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moved to combined stage.</t>
+          <t xml:space="preserve">Moved to combined stage. 21-Oct (Sam): design documentation should be attached to the MOC here.</t>
         </is>
       </c>
     </row>
@@ -43018,7 +43148,7 @@
       <c r="Y35" s="253"/>
       <c r="Z35" s="253"/>
     </row>
-    <row r="36" ht="187.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" ht="187.2" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A36" s="188">
         <v>32</v>
       </c>
@@ -43093,8 +43223,13 @@
       </c>
       <c r="Y36" s="253"/>
       <c r="Z36" s="253"/>
-    </row>
-    <row r="37" ht="230.4" x14ac:dyDescent="0.55000000000000004">
+      <c r="AA36" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21-Oct (Sam): not sure we need both 'Installation Complete?' and 'Installation Confirmed?' - keep one [TBC].</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="216.0" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A37" s="188">
         <v>33</v>
       </c>
@@ -43169,6 +43304,11 @@
       </c>
       <c r="Y37" s="253"/>
       <c r="Z37" s="253"/>
+      <c r="AA37" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[TBC] candidate for removal (see row above).</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="187.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="188">
@@ -43411,12 +43551,12 @@
       <c r="D41" s="201" t="s">
         <v>614</v>
       </c>
-      <c r="E41" s="262" t="inlineStr">
+      <c r="E41" s="263" t="inlineStr">
         <is>
           <t xml:space="preserve">Start-Up Confirmed?</t>
         </is>
       </c>
-      <c r="F41" s="263" t="inlineStr">
+      <c r="F41" s="264" t="inlineStr">
         <is>
           <t xml:space="preserve">Start-Up Confirmed?</t>
         </is>
@@ -43722,12 +43862,12 @@
       <c r="D45" s="201" t="s">
         <v>620</v>
       </c>
-      <c r="E45" s="262" t="inlineStr">
+      <c r="E45" s="263" t="inlineStr">
         <is>
           <t xml:space="preserve">Were MOC Procedures Followed?</t>
         </is>
       </c>
-      <c r="F45" s="263" t="inlineStr">
+      <c r="F45" s="264" t="inlineStr">
         <is>
           <t xml:space="preserve">Were MOC Procedures Followed?</t>
         </is>
@@ -43809,12 +43949,12 @@
       <c r="D46" s="201" t="s">
         <v>620</v>
       </c>
-      <c r="E46" s="262" t="inlineStr">
+      <c r="E46" s="263" t="inlineStr">
         <is>
           <t xml:space="preserve">MOC Process Effectiveness &amp; Feedback</t>
         </is>
       </c>
-      <c r="F46" s="263" t="inlineStr">
+      <c r="F46" s="264" t="inlineStr">
         <is>
           <t xml:space="preserve">MOC Process Effectiveness &amp; Feedback</t>
         </is>
@@ -43883,7 +44023,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" ht="28.8" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A47" s="188">
         <v>43</v>
       </c>
@@ -43954,6 +44094,11 @@
       </c>
       <c r="Y47" s="253"/>
       <c r="Z47" s="253"/>
+      <c r="AA47" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21-Oct (Sam): add questions from the MOC audit form to Follow Up (list from Sam) [TBC].</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="72.0" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A48" s="188">
@@ -44296,7 +44441,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="115.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" ht="100.8" x14ac:dyDescent="0.55000000000000004" customHeight="1">
       <c r="A52" s="188">
         <v>48</v>
       </c>
@@ -44367,8 +44512,13 @@
       </c>
       <c r="Y52" s="253"/>
       <c r="Z52" s="253"/>
-    </row>
-    <row r="53" x14ac:dyDescent="0.55000000000000004">
+      <c r="AA52" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KEEP - 21-Oct (Shaun, Hugo): traceability, e.g. phased tank works (roof removal, new roof, return to service).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" x14ac:dyDescent="0.55000000000000004" ht="86.4" customHeight="1">
       <c r="A53" s="188">
         <v>49</v>
       </c>
@@ -44391,11 +44541,19 @@
       <c r="H53" s="200" t="s">
         <v>169</v>
       </c>
-      <c r="I53" s="201"/>
+      <c r="I53" s="262" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instruction text: attach all supporting documents - risk assessment / JSA, method statement, procedures, P&amp;IDs, design documents, SDS, permits and licences.</t>
+        </is>
+      </c>
       <c r="J53" s="201" t="s">
         <v>632</v>
       </c>
-      <c r="K53" s="177"/>
+      <c r="K53" s="261" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M</t>
+        </is>
+      </c>
       <c r="L53" s="189" t="s">
         <v>14</v>
       </c>
@@ -44437,6 +44595,11 @@
       </c>
       <c r="Y53" s="253"/>
       <c r="Z53" s="253"/>
+      <c r="AA53" s="256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21-Oct (Khesar): explain under Attachments which documents are expected. Manual MOC form retired.</t>
+        </is>
+      </c>
     </row>
     <row r="54" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="188">
@@ -44783,7 +44946,7 @@
         <v>108</v>
       </c>
       <c r="G64" s="182"/>
-      <c r="H64" s="264" t="inlineStr">
+      <c r="H64" s="265" t="inlineStr">
         <is>
           <t xml:space="preserve">Lookup</t>
         </is>
@@ -44794,7 +44957,7 @@
           <t xml:space="preserve">Values: Yes / No / N/A [TBC]</t>
         </is>
       </c>
-      <c r="K64" s="265" t="inlineStr">
+      <c r="K64" s="266" t="inlineStr">
         <is>
           <t xml:space="preserve">M</t>
         </is>
@@ -49303,7 +49466,7 @@
       <c r="K168" s="59"/>
       <c r="AA168" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - object caption: 'Local Approval (Terminal Manager)'</t>
+          <t xml:space="preserve">21-Oct: Keep (functional approval). Missing: Operations, Maintenance + level approvals (TM / Regional / Global).</t>
         </is>
       </c>
     </row>
@@ -50101,7 +50264,7 @@
       <c r="K186" s="59"/>
       <c r="AA186" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - object caption: 'Regional Operations Approval'</t>
+          <t xml:space="preserve">21-Oct: Keep (functional approval). Missing: Operations, Maintenance + level approvals (TM / Regional / Global).</t>
         </is>
       </c>
     </row>
@@ -50899,7 +51062,7 @@
       <c r="K204" s="59"/>
       <c r="AA204" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - object caption: 'Global Operations Approval'</t>
+          <t xml:space="preserve">21-Oct: [TBC] re-use for a missing type - Intelex to propose. Missing: Operations, Maintenance + level approvals (TM / Regional / Global).</t>
         </is>
       </c>
     </row>
@@ -51697,7 +51860,7 @@
       <c r="K222" s="59"/>
       <c r="AA222" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - object caption: 'Global HSEC Approval'</t>
+          <t xml:space="preserve">21-Oct: [TBC] re-use for a missing type - Intelex to propose. Missing: Operations, Maintenance + level approvals (TM / Regional / Global).</t>
         </is>
       </c>
     </row>
@@ -52495,7 +52658,7 @@
       <c r="K240" s="59"/>
       <c r="AA240" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - object caption: 'Regional HSEC Approval'</t>
+          <t xml:space="preserve">21-Oct: Keep (functional approval). Missing: Operations, Maintenance + level approvals (TM / Regional / Global).</t>
         </is>
       </c>
     </row>
@@ -53293,7 +53456,7 @@
       <c r="K258" s="59"/>
       <c r="AA258" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - object caption: 'Additional Approval (ad hoc)'</t>
+          <t xml:space="preserve">21-Oct: [TBC] re-use for a missing type - Intelex to propose. Missing: Operations, Maintenance + level approvals (TM / Regional / Global).</t>
         </is>
       </c>
     </row>
@@ -55003,7 +55166,7 @@
           <t xml:space="preserve">L04 - Grade of Change</t>
         </is>
       </c>
-      <c r="K303" s="266" t="inlineStr">
+      <c r="K303" s="267" t="inlineStr">
         <is>
           <t xml:space="preserve">M</t>
         </is>
@@ -55587,7 +55750,7 @@
           <t xml:space="preserve">L04 - Grade of Change</t>
         </is>
       </c>
-      <c r="K320" s="266" t="inlineStr">
+      <c r="K320" s="267" t="inlineStr">
         <is>
           <t xml:space="preserve">M</t>
         </is>
@@ -56047,7 +56210,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M333" s="267" t="inlineStr">
+      <c r="M333" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -56057,12 +56220,12 @@
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="O333" s="267" t="inlineStr">
+      <c r="O333" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P333" s="267" t="inlineStr">
+      <c r="P333" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56172,7 +56335,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M334" s="267" t="inlineStr">
+      <c r="M334" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56182,12 +56345,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O334" s="267" t="inlineStr">
+      <c r="O334" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P334" s="267" t="inlineStr">
+      <c r="P334" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56297,7 +56460,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M335" s="267" t="inlineStr">
+      <c r="M335" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56307,12 +56470,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O335" s="267" t="inlineStr">
+      <c r="O335" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P335" s="267" t="inlineStr">
+      <c r="P335" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56422,7 +56585,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M336" s="267" t="inlineStr">
+      <c r="M336" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56432,12 +56595,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O336" s="267" t="inlineStr">
+      <c r="O336" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P336" s="267" t="inlineStr">
+      <c r="P336" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56543,7 +56706,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M337" s="267" t="inlineStr">
+      <c r="M337" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56553,12 +56716,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O337" s="267" t="inlineStr">
+      <c r="O337" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P337" s="267" t="inlineStr">
+      <c r="P337" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56660,7 +56823,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M338" s="267" t="inlineStr">
+      <c r="M338" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -56670,12 +56833,12 @@
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="O338" s="267" t="inlineStr">
+      <c r="O338" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P338" s="267" t="inlineStr">
+      <c r="P338" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56777,7 +56940,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M339" s="267" t="inlineStr">
+      <c r="M339" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -56787,12 +56950,12 @@
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="O339" s="267" t="inlineStr">
+      <c r="O339" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P339" s="267" t="inlineStr">
+      <c r="P339" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56898,7 +57061,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M340" s="267" t="inlineStr">
+      <c r="M340" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -56908,12 +57071,12 @@
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="O340" s="267" t="inlineStr">
+      <c r="O340" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P340" s="267" t="inlineStr">
+      <c r="P340" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -56964,7 +57127,7 @@
         </is>
       </c>
     </row>
-    <row r="341" x14ac:dyDescent="0.55000000000000004" ht="86.4" customHeight="1">
+    <row r="341" x14ac:dyDescent="0.55000000000000004" ht="115.2" customHeight="1">
       <c r="A341" s="253">
         <v>9</v>
       </c>
@@ -56989,12 +57152,12 @@
       </c>
       <c r="E341" s="257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Action Plans</t>
+          <t xml:space="preserve">Action Plans (OPTIONAL)</t>
         </is>
       </c>
       <c r="F341" s="257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Action Plans</t>
+          <t xml:space="preserve">Action Plans (OPTIONAL)</t>
         </is>
       </c>
       <c r="G341" s="254" t="inlineStr">
@@ -57010,7 +57173,7 @@
       <c r="I341" s="254"/>
       <c r="J341" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">1:M relation to Action Plan object; columns: Action No. | Description | Person Responsible | Due Date | Status. [Intelex to confirm]</t>
+          <t xml:space="preserve">1:M relation to Action Plan object; columns: Action No. | Description | Person Responsible | Due Date | Status. Only if Intelex confirms low effort. Decision 21-Oct: MOC Tasks remain the MOC actions.</t>
         </is>
       </c>
       <c r="K341" s="256" t="inlineStr">
@@ -57023,7 +57186,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M341" s="267" t="inlineStr">
+      <c r="M341" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -57033,12 +57196,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O341" s="267" t="inlineStr">
+      <c r="O341" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P341" s="267" t="inlineStr">
+      <c r="P341" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -57085,17 +57248,17 @@
       </c>
       <c r="AA341" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alonso / Sam: traceability of actions back to the MOC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="342" ht="57.6" customHeight="1">
+          <t xml:space="preserve">Nice-to-have (Sam). Shaun 21-Oct: OK with tasks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="342" ht="72.0" customHeight="1">
       <c r="A342" s="253">
         <v>10</v>
       </c>
       <c r="B342" s="255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Initiation</t>
+          <t xml:space="preserve">Draft (MOC Task)</t>
         </is>
       </c>
       <c r="C342" s="255" t="inlineStr">
@@ -57105,37 +57268,37 @@
       </c>
       <c r="D342" s="255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Initiation Information Details</t>
+          <t xml:space="preserve">MOC Task Details</t>
         </is>
       </c>
       <c r="E342" s="257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Change Owner</t>
+          <t xml:space="preserve">Complete Before Stage</t>
         </is>
       </c>
       <c r="F342" s="257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Change Owner</t>
+          <t xml:space="preserve">Complete Before Stage</t>
         </is>
       </c>
       <c r="G342" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accountable for the change through to closure.</t>
+          <t xml:space="preserve">MOC stage by which the task must be closed.</t>
         </is>
       </c>
       <c r="H342" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relations</t>
+          <t xml:space="preserve">Lookup (Approval / Start Up / Follow Up)</t>
         </is>
       </c>
       <c r="I342" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tooltip: Person accountable for the change until closure (may be the requester).</t>
+          <t xml:space="preserve">Tooltip: Pre-startup tasks = Start Up; post-change tasks (e.g. P&amp;ID update) = Follow Up.</t>
         </is>
       </c>
       <c r="J342" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">M:1 relation to Employee. Default Value: Change Requester.</t>
+          <t xml:space="preserve">Field on MOC Task (all task types). MOC stage gate checks only open tasks due for that stage [Intelex to confirm].</t>
         </is>
       </c>
       <c r="K342" s="256" t="inlineStr">
@@ -57148,9 +57311,9 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M342" s="267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Y</t>
+      <c r="M342" s="268" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="N342" s="253" t="inlineStr">
@@ -57158,12 +57321,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O342" s="267" t="inlineStr">
+      <c r="O342" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P342" s="267" t="inlineStr">
+      <c r="P342" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -57175,7 +57338,7 @@
       </c>
       <c r="R342" s="253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Y</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="S342" s="253" t="inlineStr">
@@ -57185,7 +57348,7 @@
       </c>
       <c r="T342" s="253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Y</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="U342" s="253" t="inlineStr">
@@ -57195,7 +57358,7 @@
       </c>
       <c r="V342" s="253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Y</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="W342" s="253" t="inlineStr">
@@ -57205,16 +57368,16 @@
       </c>
       <c r="X342" s="253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Y</t>
+          <t xml:space="preserve">N</t>
         </is>
       </c>
       <c r="AA342" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">BRD FR-B3-026 (Should) / FR-B3-004: originator vs owner.</t>
-        </is>
-      </c>
-    </row>
-    <row r="343" ht="43.2" customHeight="1">
+          <t xml:space="preserve">21-Oct (Khesar / Sam): tasks due later must not block the MOC. BRD FR-B3-032.</t>
+        </is>
+      </c>
+    </row>
+    <row r="343" ht="57.6" customHeight="1">
       <c r="A343" s="253">
         <v>11</v>
       </c>
@@ -57235,17 +57398,17 @@
       </c>
       <c r="E343" s="257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operational Owner</t>
+          <t xml:space="preserve">Change Owner</t>
         </is>
       </c>
       <c r="F343" s="257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operational Owner</t>
+          <t xml:space="preserve">Change Owner</t>
         </is>
       </c>
       <c r="G343" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner of the affected area or asset.</t>
+          <t xml:space="preserve">Accountable for the change through to closure.</t>
         </is>
       </c>
       <c r="H343" s="254" t="inlineStr">
@@ -57255,12 +57418,12 @@
       </c>
       <c r="I343" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tooltip: Responsible for operational readiness before start-up.</t>
+          <t xml:space="preserve">Tooltip: Person accountable for the change until closure (may be the requester).</t>
         </is>
       </c>
       <c r="J343" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">M:1 relation to Employee.</t>
+          <t xml:space="preserve">M:1 relation to Employee. Default Value: Change Requester.</t>
         </is>
       </c>
       <c r="K343" s="256" t="inlineStr">
@@ -57273,7 +57436,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M343" s="267" t="inlineStr">
+      <c r="M343" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -57283,12 +57446,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O343" s="267" t="inlineStr">
+      <c r="O343" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P343" s="267" t="inlineStr">
+      <c r="P343" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -57335,11 +57498,11 @@
       </c>
       <c r="AA343" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">BRD FR-B3-004 (Must).</t>
-        </is>
-      </c>
-    </row>
-    <row r="344" ht="57.6" customHeight="1">
+          <t xml:space="preserve">BRD FR-B3-026 (Should) / FR-B3-004: originator vs owner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="344" ht="43.2" customHeight="1">
       <c r="A344" s="253">
         <v>12</v>
       </c>
@@ -57360,32 +57523,32 @@
       </c>
       <c r="E344" s="257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reason for Change &amp; Technical Basis</t>
+          <t xml:space="preserve">Operational Owner</t>
         </is>
       </c>
       <c r="F344" s="257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reason for Change &amp; Technical Basis</t>
+          <t xml:space="preserve">Operational Owner</t>
         </is>
       </c>
       <c r="G344" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Detailed justification.</t>
+          <t xml:space="preserve">Owner of the affected area or asset.</t>
         </is>
       </c>
       <c r="H344" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text (multi-line)</t>
+          <t xml:space="preserve">Relations</t>
         </is>
       </c>
       <c r="I344" s="254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tooltip: Why the change is needed, technical basis, scope and current situation.</t>
+          <t xml:space="preserve">Tooltip: Responsible for operational readiness before start-up.</t>
         </is>
       </c>
       <c r="J344" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">No length limit.</t>
+          <t xml:space="preserve">M:1 relation to Employee.</t>
         </is>
       </c>
       <c r="K344" s="256" t="inlineStr">
@@ -57398,7 +57561,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M344" s="267" t="inlineStr">
+      <c r="M344" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -57408,12 +57571,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O344" s="267" t="inlineStr">
+      <c r="O344" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P344" s="267" t="inlineStr">
+      <c r="P344" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -57460,7 +57623,7 @@
       </c>
       <c r="AA344" s="256" t="inlineStr">
         <is>
-          <t xml:space="preserve">BRD FR-B3-001 (Must); Change Description is limited to 255 characters.</t>
+          <t xml:space="preserve">BRD FR-B3-004 (Must).</t>
         </is>
       </c>
     </row>
@@ -57515,7 +57678,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M345" s="267" t="inlineStr">
+      <c r="M345" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -57525,12 +57688,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O345" s="267" t="inlineStr">
+      <c r="O345" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P345" s="267" t="inlineStr">
+      <c r="P345" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -57636,7 +57799,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M346" s="267" t="inlineStr">
+      <c r="M346" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -57646,12 +57809,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O346" s="267" t="inlineStr">
+      <c r="O346" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P346" s="267" t="inlineStr">
+      <c r="P346" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -57761,7 +57924,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M347" s="267" t="inlineStr">
+      <c r="M347" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -57771,12 +57934,12 @@
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="O347" s="267" t="inlineStr">
+      <c r="O347" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P347" s="267" t="inlineStr">
+      <c r="P347" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -57882,7 +58045,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M348" s="267" t="inlineStr">
+      <c r="M348" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -57892,12 +58055,12 @@
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="O348" s="267" t="inlineStr">
+      <c r="O348" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P348" s="267" t="inlineStr">
+      <c r="P348" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58003,7 +58166,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M349" s="267" t="inlineStr">
+      <c r="M349" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58013,12 +58176,12 @@
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="O349" s="267" t="inlineStr">
+      <c r="O349" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P349" s="267" t="inlineStr">
+      <c r="P349" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
@@ -58120,7 +58283,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M350" s="267" t="inlineStr">
+      <c r="M350" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58130,12 +58293,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O350" s="267" t="inlineStr">
+      <c r="O350" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="P350" s="267" t="inlineStr">
+      <c r="P350" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58241,7 +58404,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M351" s="267" t="inlineStr">
+      <c r="M351" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58251,12 +58414,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O351" s="267" t="inlineStr">
+      <c r="O351" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="P351" s="267" t="inlineStr">
+      <c r="P351" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58358,7 +58521,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M352" s="267" t="inlineStr">
+      <c r="M352" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58368,12 +58531,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O352" s="267" t="inlineStr">
+      <c r="O352" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P352" s="267" t="inlineStr">
+      <c r="P352" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58475,7 +58638,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M353" s="267" t="inlineStr">
+      <c r="M353" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58485,12 +58648,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O353" s="267" t="inlineStr">
+      <c r="O353" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P353" s="267" t="inlineStr">
+      <c r="P353" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58592,7 +58755,7 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="M354" s="267" t="inlineStr">
+      <c r="M354" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -58602,12 +58765,12 @@
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="O354" s="267" t="inlineStr">
+      <c r="O354" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
       </c>
-      <c r="P354" s="267" t="inlineStr">
+      <c r="P354" s="268" t="inlineStr">
         <is>
           <t xml:space="preserve">N</t>
         </is>
@@ -63926,7 +64089,7 @@
         <v>387</v>
       </c>
       <c r="B4" s="74"/>
-      <c r="C4" s="268" t="inlineStr">
+      <c r="C4" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">R - Priority field removed (Grade of Change is the single driver).</t>
         </is>
@@ -63977,7 +64140,7 @@
         <v>190</v>
       </c>
       <c r="B11" s="74"/>
-      <c r="C11" s="268" t="inlineStr">
+      <c r="C11" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Check: values are the Approval objects (same as L07); Task Type should list MOC Task children (L06). Intelex to confirm.</t>
         </is>
@@ -64060,7 +64223,7 @@
         <v>197</v>
       </c>
       <c r="B20" s="74"/>
-      <c r="C20" s="268" t="inlineStr">
+      <c r="C20" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">M - aligned to the new 6-stage workflow.</t>
         </is>
@@ -64089,12 +64252,12 @@
       <c r="E22" s="13"/>
     </row>
     <row r="23" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="268" t="inlineStr">
+      <c r="A23" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
-      <c r="B23" s="268" t="inlineStr">
+      <c r="B23" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Evaluation, Design &amp; Analysis</t>
         </is>
@@ -64103,12 +64266,12 @@
       <c r="E23" s="13"/>
     </row>
     <row r="24" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="269" t="inlineStr">
+      <c r="A24" s="270" t="inlineStr">
         <is>
           <t xml:space="preserve">Approval</t>
         </is>
       </c>
-      <c r="B24" s="269" t="inlineStr">
+      <c r="B24" s="270" t="inlineStr">
         <is>
           <t xml:space="preserve">Approval</t>
         </is>
@@ -64117,12 +64280,12 @@
       <c r="E24" s="13"/>
     </row>
     <row r="25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="269" t="inlineStr">
+      <c r="A25" s="270" t="inlineStr">
         <is>
           <t xml:space="preserve">Implementation</t>
         </is>
       </c>
-      <c r="B25" s="269" t="inlineStr">
+      <c r="B25" s="270" t="inlineStr">
         <is>
           <t xml:space="preserve">Implementation</t>
         </is>
@@ -64131,12 +64294,12 @@
       <c r="E25" s="13"/>
     </row>
     <row r="26" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="269" t="inlineStr">
+      <c r="A26" s="270" t="inlineStr">
         <is>
           <t xml:space="preserve">Start-Up</t>
         </is>
       </c>
-      <c r="B26" s="269" t="inlineStr">
+      <c r="B26" s="270" t="inlineStr">
         <is>
           <t xml:space="preserve">Start-Up</t>
         </is>
@@ -64145,12 +64308,12 @@
       <c r="E26" s="13"/>
     </row>
     <row r="27" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="269" t="inlineStr">
+      <c r="A27" s="270" t="inlineStr">
         <is>
           <t xml:space="preserve">Follow-Up</t>
         </is>
       </c>
-      <c r="B27" s="269" t="inlineStr">
+      <c r="B27" s="270" t="inlineStr">
         <is>
           <t xml:space="preserve">Follow-Up</t>
         </is>
@@ -64159,17 +64322,17 @@
       <c r="E27" s="13"/>
     </row>
     <row r="28" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="269"/>
-      <c r="B28" s="269"/>
+      <c r="A28" s="270"/>
+      <c r="B28" s="270"/>
     </row>
     <row r="30" ht="43.2" x14ac:dyDescent="0.85" customHeight="1">
-      <c r="A30" s="270" t="inlineStr">
+      <c r="A30" s="271" t="inlineStr">
         <is>
           <t xml:space="preserve">L04 - Grade of Change (Change Impact)</t>
         </is>
       </c>
       <c r="B30" s="74"/>
-      <c r="C30" s="268" t="inlineStr">
+      <c r="C30" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">M - single criticality list used by MOC and by Screening / Task / Approval setups. Minor = Local, Moderate = Regional, Major = Global approval.</t>
         </is>
@@ -64184,36 +64347,36 @@
       </c>
     </row>
     <row r="32" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="268" t="inlineStr">
+      <c r="A32" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
-      <c r="B32" s="268" t="inlineStr">
+      <c r="B32" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Minor</t>
         </is>
       </c>
     </row>
     <row r="33" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="268" t="inlineStr">
+      <c r="A33" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate</t>
         </is>
       </c>
-      <c r="B33" s="268" t="inlineStr">
+      <c r="B33" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate</t>
         </is>
       </c>
     </row>
     <row r="34" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="269" t="inlineStr">
+      <c r="A34" s="270" t="inlineStr">
         <is>
           <t xml:space="preserve">Major</t>
         </is>
       </c>
-      <c r="B34" s="269" t="inlineStr">
+      <c r="B34" s="270" t="inlineStr">
         <is>
           <t xml:space="preserve">Major</t>
         </is>
@@ -64224,7 +64387,7 @@
         <v>382</v>
       </c>
       <c r="B36" s="74"/>
-      <c r="C36" s="268" t="inlineStr">
+      <c r="C36" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">R - duplicate of L01; replace its references (Task/Approval setup, Change Impact) by L04.</t>
         </is>
@@ -64267,7 +64430,7 @@
         <v>447</v>
       </c>
       <c r="B42" s="74"/>
-      <c r="C42" s="268" t="inlineStr">
+      <c r="C42" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Keep. Mapping to checklist sections: Impact/Hazard Assessment (B), Process (C, E-H), Documentation (D), Training + Change Communication (I), PSSR (K), Checklist (generic).</t>
         </is>
@@ -64337,14 +64500,14 @@
         <v>196</v>
       </c>
     </row>
-    <row r="52" ht="28.8" x14ac:dyDescent="0.85" customHeight="1">
+    <row r="52" ht="72.0" x14ac:dyDescent="0.85" customHeight="1">
       <c r="A52" s="61" t="s">
         <v>769</v>
       </c>
       <c r="B52" s="74"/>
-      <c r="C52" s="268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M - captions only (existing approval objects re-used for Local / Regional / Global levels).</t>
+      <c r="C52" s="269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[TBC] 21-Oct: keep OOTB types for functional approvals; add Operations (Khesar) and Maintenance; level approvals (TM / Regional HSEC-Ops / Global HSEC-Ops) also needed. Intelex to propose re-caption vs new objects.</t>
         </is>
       </c>
     </row>
@@ -64360,60 +64523,48 @@
       <c r="A54" s="13" t="s">
         <v>418</v>
       </c>
-      <c r="B54" s="268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Regional Operations Approval</t>
-        </is>
+      <c r="B54" s="13" t="s">
+        <v>419</v>
       </c>
     </row>
     <row r="55" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="13" t="s">
         <v>420</v>
       </c>
-      <c r="B55" s="268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Regional HSEC Approval</t>
-        </is>
+      <c r="B55" s="13" t="s">
+        <v>421</v>
       </c>
     </row>
     <row r="56" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" t="s">
         <v>422</v>
       </c>
-      <c r="B56" s="269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Local Approval (Terminal Manager)</t>
-        </is>
+      <c r="B56" t="s">
+        <v>423</v>
       </c>
     </row>
     <row r="57" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" t="s">
         <v>424</v>
       </c>
-      <c r="B57" s="269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Global HSEC Approval</t>
-        </is>
+      <c r="B57" t="s">
+        <v>425</v>
       </c>
     </row>
     <row r="58" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" t="s">
         <v>426</v>
       </c>
-      <c r="B58" s="269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Global Operations Approval</t>
-        </is>
+      <c r="B58" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="59" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" t="s">
         <v>428</v>
       </c>
-      <c r="B59" s="269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Additional Approval (ad hoc)</t>
-        </is>
+      <c r="B59" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="62">
@@ -64422,7 +64573,7 @@
           <t xml:space="preserve">L08 - Type of Change (MOC Category data)</t>
         </is>
       </c>
-      <c r="C62" s="268" t="inlineStr">
+      <c r="C62" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">A - records of the MOC Category object (caption 'Type of Change').</t>
         </is>
@@ -64441,96 +64592,96 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="268" t="inlineStr">
+      <c r="A64" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Change of Design / Equipment</t>
         </is>
       </c>
-      <c r="B64" s="271" t="inlineStr">
+      <c r="B64" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Change of Design / Equipment</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="268" t="inlineStr">
+      <c r="A65" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">2. Change of Process</t>
         </is>
       </c>
-      <c r="B65" s="271" t="inlineStr">
+      <c r="B65" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">2. Change of Process</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="268" t="inlineStr">
+      <c r="A66" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">3. Change of Procedure</t>
         </is>
       </c>
-      <c r="B66" s="271" t="inlineStr">
+      <c r="B66" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">3. Change of Procedure</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="268" t="inlineStr">
+      <c r="A67" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">4. Change of Control Systems / IT / SIS</t>
         </is>
       </c>
-      <c r="B67" s="271" t="inlineStr">
+      <c r="B67" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">4. Change of Control Systems / IT / SIS</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="268" t="inlineStr">
+      <c r="A68" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">5. Organisational / Personnel Change</t>
         </is>
       </c>
-      <c r="B68" s="271" t="inlineStr">
+      <c r="B68" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">5. Organisational / Personnel Change</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="268" t="inlineStr">
+      <c r="A69" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">6. Temporary Change</t>
         </is>
       </c>
-      <c r="B69" s="271" t="inlineStr">
+      <c r="B69" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">6. Temporary Change</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="268" t="inlineStr">
+      <c r="A70" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">7. Regulatory / Permit-Driven Change</t>
         </is>
       </c>
-      <c r="B70" s="271" t="inlineStr">
+      <c r="B70" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">7. Regulatory / Permit-Driven Change</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="268" t="inlineStr">
+      <c r="A71" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">8. Changes to Utility &amp; HSE Protection Systems</t>
         </is>
       </c>
-      <c r="B71" s="271" t="inlineStr">
+      <c r="B71" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">8. Changes to Utility &amp; HSE Protection Systems</t>
         </is>
@@ -64566,176 +64717,176 @@
       </c>
     </row>
     <row r="76" ht="144.0" customHeight="1">
-      <c r="A76" s="268" t="inlineStr">
+      <c r="A76" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Change of Design / Equipment</t>
         </is>
       </c>
-      <c r="B76" s="268" t="inlineStr">
+      <c r="B76" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Replace for an identical one. Replacement by an identical component with the same engineering specifications, construction material, and design range. Includes relocation of equipment within the same service and operating conditions</t>
         </is>
       </c>
-      <c r="C76" s="268" t="inlineStr">
+      <c r="C76" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Replace for a similar one. Replacement by a functionally similar component; may differ in brand or model but remains within the same design range. Includes relocation to a different service or operating environment, or decommissioning of non-safety-critical equipment</t>
         </is>
       </c>
-      <c r="D76" s="268" t="inlineStr">
+      <c r="D76" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Replace for a different one. Technologically different component, different construction material, or outside the original design range. Includes any departure from original design intent, decommissioning of safety-critical equipment, or permanent removal of equipment with associated safeguard implications</t>
         </is>
       </c>
     </row>
     <row r="77" ht="144.0" customHeight="1">
-      <c r="A77" s="268" t="inlineStr">
+      <c r="A77" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">2. Change of Process</t>
         </is>
       </c>
-      <c r="B77" s="268" t="inlineStr">
+      <c r="B77" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Change of environment. Process carried out in same-size equipment with same construction materials and instrumentation. Capacity change ≤ 10%. Substitution of a non-hazardous material with an equivalent; no change to process parameters</t>
         </is>
       </c>
-      <c r="C77" s="268" t="inlineStr">
+      <c r="C77" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Change of scale. Capacity change &gt; 10% in volume, weight, or flow. Substitution of a hazardous material (Risk Class ≥ 3) with an equivalent within the same risk class and quantity variation ≤ 20%. Modifications to process systems (vessels, piping, relief devices) within existing design parameters</t>
         </is>
       </c>
-      <c r="D77" s="268" t="inlineStr">
+      <c r="D77" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Change of conditions. a) New process or component; b) New hazardous materials not currently present; c) Change of any process parameter that affects system integrity, the Safe Operating Envelope, or existing safeguards; d) Modifications to process systems (vessels, piping, relief devices) outside existing design parameters or affecting safeguard integrity</t>
         </is>
       </c>
     </row>
     <row r="78" ht="86.4" customHeight="1">
-      <c r="A78" s="268" t="inlineStr">
+      <c r="A78" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">3. Change of Procedure</t>
         </is>
       </c>
-      <c r="B78" s="268" t="inlineStr">
+      <c r="B78" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Minor update. Editorial correction or clarification of an existing procedure with no change to operational sequence, frequency, or responsibilities</t>
         </is>
       </c>
-      <c r="C78" s="268" t="inlineStr">
+      <c r="C78" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Operational modification. Change of sequence, frequency, or responsible party in a key operational, maintenance, or emergency response procedure</t>
         </is>
       </c>
-      <c r="D78" s="268" t="inlineStr">
+      <c r="D78" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">New procedure or elimination of control. Creation of a procedure for a previously undefined operation, or removal of an existing safety critical control step. Includes changes to emergency response plans</t>
         </is>
       </c>
     </row>
     <row r="79" ht="86.4" customHeight="1">
-      <c r="A79" s="268" t="inlineStr">
+      <c r="A79" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">4. Change of Control Systems / IT / SIS</t>
         </is>
       </c>
-      <c r="B79" s="268" t="inlineStr">
+      <c r="B79" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Configuration change. Minor adjustment to alarm setpoints or display parameters within approved operating ranges; no change to logic or interlocks</t>
         </is>
       </c>
-      <c r="C79" s="268" t="inlineStr">
+      <c r="C79" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Software or logic modification. Modification to control system logic, PLC/DCS programming, or alarm management system; no change to SIS/SIL functions</t>
         </is>
       </c>
-      <c r="D79" s="268" t="inlineStr">
+      <c r="D79" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Safety system modification. Any change to Safety Instrumented Systems (SIS/SIL), emergency shutdown systems, or IT/OT systems that interface with safety-critical functions; or introduction of new control system architecture</t>
         </is>
       </c>
     </row>
     <row r="80" ht="86.4" customHeight="1">
-      <c r="A80" s="268" t="inlineStr">
+      <c r="A80" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">5. Organisational / Personnel Change</t>
         </is>
       </c>
-      <c r="B80" s="268" t="inlineStr">
+      <c r="B80" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Minor role change. Temporary reassignment of an operator within the same competency level, with no impact on critical safety roles or staffing levels</t>
         </is>
       </c>
-      <c r="C80" s="268" t="inlineStr">
+      <c r="C80" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Change of area responsible. Change of supervisor, coordinator, or key contractor in an operational area; safety-critical roles remain filled by competent personnel</t>
         </is>
       </c>
-      <c r="D80" s="268" t="inlineStr">
+      <c r="D80" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Loss or change of critical competency. Team restructuring, contractor change-out, or reduction of staffing in a risk-critical area. Includes situations where inexperienced personnel assume critical decision-making roles</t>
         </is>
       </c>
     </row>
     <row r="81" ht="129.6" customHeight="1">
-      <c r="A81" s="268" t="inlineStr">
+      <c r="A81" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">6. Temporary Change</t>
         </is>
       </c>
-      <c r="B81" s="268" t="inlineStr">
+      <c r="B81" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Short duration, low risk. Fully reversible, no impact on safeguards or safety-critical systems. Includes installation of temporary equipment with no safeguard implications. Removal date defined prior to implementation</t>
         </is>
       </c>
-      <c r="C81" s="268" t="inlineStr">
+      <c r="C81" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Extended duration, moderate risk. Reversible, with defined monitoring plan, removal date, and re-approval authority. Includes temporary equipment that affects operating procedures or non-safety-critical instrumentation. Scope clearly bounded and documented</t>
         </is>
       </c>
-      <c r="D81" s="268" t="inlineStr">
+      <c r="D81" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Safeguard-affecting. Any duration if it affects safety devices, alarms, interlocks, or passive safeguards. Includes installation or removal of temporary equipment that bypasses or impairs any safeguard. Scope or duration must not be exceeded without formal review and re-approval</t>
         </is>
       </c>
     </row>
     <row r="82" ht="72.0" customHeight="1">
-      <c r="A82" s="268" t="inlineStr">
+      <c r="A82" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">7. Regulatory / Permit-Driven Change</t>
         </is>
       </c>
-      <c r="B82" s="268" t="inlineStr">
+      <c r="B82" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Administrative update. Change requires notification to a regulatory body but no amendment to existing permits or licences</t>
         </is>
       </c>
-      <c r="C82" s="268" t="inlineStr">
+      <c r="C82" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Permit amendment. Change requires amendment to one or more existing environmental or operating permits</t>
         </is>
       </c>
-      <c r="D82" s="268" t="inlineStr">
+      <c r="D82" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">New permit or consent required. Change requires a new licence, permit, or regulatory consent (e.g. Environmental Permit, HSE Reports, Hazardous Substances Consent) prior to implementation</t>
         </is>
       </c>
     </row>
     <row r="83" ht="144.0" customHeight="1">
-      <c r="A83" s="268" t="inlineStr">
+      <c r="A83" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">8. Changes to Utility &amp; HSE Protection Systems</t>
         </is>
       </c>
-      <c r="B83" s="268" t="inlineStr">
+      <c r="B83" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Minor adjustment. Modification to utility systems (steam, air, nitrogen, water) or HSE protection infrastructure (bunding, drainage, fire suppression, gas detection) within existing design parameters and with no reduction in protection standard</t>
         </is>
       </c>
-      <c r="C83" s="268" t="inlineStr">
+      <c r="C83" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate modification. Change to utility systems or HSE protection infrastructure that temporarily reduces protection standard but with compensatory measures defined and in place; or change that requires review and update of inspection or maintenance schedules</t>
         </is>
       </c>
-      <c r="D83" s="268" t="inlineStr">
+      <c r="D83" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Significant modification or removal. Change that permanently reduces the standard of HSE protection (e.g. reduction in bund capacity, removal or relocation of gas detection, modification to fire suppression coverage); or change to utility systems that affects the operability of safety-critical equipment</t>
         </is>
@@ -64749,35 +64900,35 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="268" t="inlineStr">
+      <c r="A86" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Landing of a floating deck / roof (IFR landing)</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="268" t="inlineStr">
+      <c r="A87" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Tank entry</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="268" t="inlineStr">
+      <c r="A88" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Any change to Safety Critical Equipment purchasing, maintenance or spares holding</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="268" t="inlineStr">
+      <c r="A89" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Safety Critical Equipment out of service / safeguard bypassed (any duration)</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="268" t="inlineStr">
+      <c r="A90" s="269" t="inlineStr">
         <is>
           <t xml:space="preserve">Over-capacity of a dry bulk terminal [TBC]</t>
         </is>

</xml_diff>

<commit_message>
Redraw MOC workflow diagram as Impala TO-BE and embed it in the workbook
The OOTB Visio object on the Workflow sheet is replaced by the TO-BE
diagram (6 stages, emergency path, roll back, cancel, stage notes per
MOC Proposal Rev2). PNG and editable SVG added to docs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018d6Sqji3PhM1w1Xd54RvCw
</commit_message>
<xml_diff>
--- a/docs/moc/Impala - Configuration Workbook - Management of Change v1.2 (Impala requirements DRAFT).xlsx
+++ b/docs/moc/Impala - Configuration Workbook - Management of Change v1.2 (Impala requirements DRAFT).xlsx
@@ -28352,61 +28352,6 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>0</xdr:col>
-          <xdr:colOff>0</xdr:colOff>
-          <xdr:row>22</xdr:row>
-          <xdr:rowOff>99060</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>9</xdr:col>
-          <xdr:colOff>495300</xdr:colOff>
-          <xdr:row>64</xdr:row>
-          <xdr:rowOff>22860</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2049" name="Object 1" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s2049"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000001080000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-            </a:solidFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a:ln>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -28575,6 +28520,39 @@
     </mc:Choice>
     <mc:Fallback/>
   </mc:AlternateContent>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="18097500" cy="7077075"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3001" name="Impala MOC Workflow TO-BE" descr="MOC workflow - Impala proposal (TO-BE), MOC Proposal Rev2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="18097500" cy="7077075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -37274,7 +37252,7 @@
       </c>
       <c r="J68" s="239" t="inlineStr">
         <is>
-          <t xml:space="preserve">M - Impala proposal (internal pre-design 20-Oct-2026, 'MOC Proposal.xlsx'). 6 stages instead of 7. Replacement in Kind path ON HOLD: may be re-used as the 'Simplified MOC' route [TBC]. The diagram above shows the OOTB workflow and must be redrawn by Intelex.</t>
+          <t xml:space="preserve">M - Impala proposal (internal pre-design 20-Oct-2026, 'MOC Proposal.xlsx'). 6 stages instead of 7. Replacement in Kind re-used as 'Simple Change?' (same workflow, no checklist). The diagram above has been redrawn by Impala as the TO-BE workflow (replaces the OOTB Visio); Intelex may re-draw it in Visio.</t>
         </is>
       </c>
     </row>
@@ -37984,31 +37962,6 @@
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
   <oleObjects>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice Requires="x14">
-        <oleObject progId="Visio.Drawing.15" shapeId="2049" r:id="rId4">
-          <objectPr defaultSize="0" autoPict="0" r:id="rId5">
-            <anchor moveWithCells="1">
-              <from>
-                <xdr:col>0</xdr:col>
-                <xdr:colOff>0</xdr:colOff>
-                <xdr:row>22</xdr:row>
-                <xdr:rowOff>99060</xdr:rowOff>
-              </from>
-              <to>
-                <xdr:col>9</xdr:col>
-                <xdr:colOff>495300</xdr:colOff>
-                <xdr:row>64</xdr:row>
-                <xdr:rowOff>22860</xdr:rowOff>
-              </to>
-            </anchor>
-          </objectPr>
-        </oleObject>
-      </mc:Choice>
-      <mc:Fallback>
-        <oleObject progId="Visio.Drawing.15" shapeId="2049" r:id="rId4"/>
-      </mc:Fallback>
-    </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
         <oleObject progId="Visio.Drawing.15" shapeId="2050" r:id="rId6">

</xml_diff>